<commit_message>
fortificant for iron changed to NaFeEDTA
</commit_message>
<xml_diff>
--- a/data/processed/india_rice_inad.xlsx
+++ b/data/processed/india_rice_inad.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wfp-my.sharepoint.com/personal/gabriel_battcock_wfp_org/Documents/Documents/MIMI_mac/nsso_hces_2023/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{2EF4D3E4-EF52-4F5B-BB4E-507D01FBBE94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC5FF6A6-90B8-4FA2-BE3C-604E8A19A0C3}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{2EF4D3E4-EF52-4F5B-BB4E-507D01FBBE94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40D35511-8D7A-491A-B3F1-28734E3BDA96}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="-15870" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="india_rice_inad" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="79">
   <si>
     <t>category</t>
   </si>
@@ -759,10 +760,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -12338,4 +12340,4088 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C74A6C3E-28C0-4B7B-9601-0E9B64F5F4A6}">
+  <dimension ref="A1:X55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="16384" width="8.7265625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="W1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
+        <v>45.865506961097502</v>
+      </c>
+      <c r="B2" s="3">
+        <v>40.569909885203799</v>
+      </c>
+      <c r="C2" s="3">
+        <v>16.588401693200499</v>
+      </c>
+      <c r="D2" s="3">
+        <v>46.204625678266197</v>
+      </c>
+      <c r="E2" s="3">
+        <v>43.520127752523898</v>
+      </c>
+      <c r="F2" s="3">
+        <v>23.050757445545699</v>
+      </c>
+      <c r="G2" s="3">
+        <v>68.986169096299193</v>
+      </c>
+      <c r="H2" s="3">
+        <v>52.034134869504598</v>
+      </c>
+      <c r="I2" s="3">
+        <v>40.105706253207799</v>
+      </c>
+      <c r="J2" s="3">
+        <v>97.448828726615105</v>
+      </c>
+      <c r="K2" s="3">
+        <v>94.296763991185202</v>
+      </c>
+      <c r="L2" s="3">
+        <v>80.582976989776299</v>
+      </c>
+      <c r="M2" s="3">
+        <v>36.061275579399698</v>
+      </c>
+      <c r="N2" s="3">
+        <v>24.998063913519498</v>
+      </c>
+      <c r="O2" s="3">
+        <v>11.833881292664</v>
+      </c>
+      <c r="P2" s="3">
+        <v>85.384673704236704</v>
+      </c>
+      <c r="Q2" s="3">
+        <v>71.729298323531495</v>
+      </c>
+      <c r="R2" s="3">
+        <v>41.850456687262401</v>
+      </c>
+      <c r="S2" s="3">
+        <v>92.985845725084801</v>
+      </c>
+      <c r="T2" s="3">
+        <v>84.652408404543095</v>
+      </c>
+      <c r="U2" s="3">
+        <v>58.396862832095302</v>
+      </c>
+      <c r="V2" s="3">
+        <v>85.313837451210802</v>
+      </c>
+      <c r="W2" s="3">
+        <v>76.629985471518594</v>
+      </c>
+      <c r="X2" s="3">
+        <v>40.929708912701898</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>27.099296678326699</v>
+      </c>
+      <c r="B3" s="3">
+        <v>21.964725770321099</v>
+      </c>
+      <c r="C3" s="3">
+        <v>7.2415781875958602</v>
+      </c>
+      <c r="D3" s="3">
+        <v>14.1148785751669</v>
+      </c>
+      <c r="E3" s="3">
+        <v>12.6455526219686</v>
+      </c>
+      <c r="F3" s="3">
+        <v>7.8576285044860397</v>
+      </c>
+      <c r="G3" s="3">
+        <v>72.161947904869805</v>
+      </c>
+      <c r="H3" s="3">
+        <v>52.2024348810872</v>
+      </c>
+      <c r="I3" s="3">
+        <v>38.158267270668198</v>
+      </c>
+      <c r="J3" s="3">
+        <v>91.688867941084197</v>
+      </c>
+      <c r="K3" s="3">
+        <v>84.467099848937707</v>
+      </c>
+      <c r="L3" s="3">
+        <v>64.257835136337107</v>
+      </c>
+      <c r="M3" s="3">
+        <v>17.7029504390493</v>
+      </c>
+      <c r="N3" s="3">
+        <v>7.0448967358115802</v>
+      </c>
+      <c r="O3" s="3">
+        <v>4.0340933823270504</v>
+      </c>
+      <c r="P3" s="3">
+        <v>87.591836680975803</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>72.589075249983907</v>
+      </c>
+      <c r="R3" s="3">
+        <v>39.018950758795</v>
+      </c>
+      <c r="S3" s="3">
+        <v>94.151123676332801</v>
+      </c>
+      <c r="T3" s="3">
+        <v>84.114442710538398</v>
+      </c>
+      <c r="U3" s="3">
+        <v>51.962805740580301</v>
+      </c>
+      <c r="V3" s="3">
+        <v>86.444967889397304</v>
+      </c>
+      <c r="W3" s="3">
+        <v>73.796276748935696</v>
+      </c>
+      <c r="X3" s="3">
+        <v>34.3058924792197</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
+        <v>17.049636337717001</v>
+      </c>
+      <c r="B4" s="3">
+        <v>15.907737111109601</v>
+      </c>
+      <c r="C4" s="3">
+        <v>11.768372863862099</v>
+      </c>
+      <c r="D4" s="3">
+        <v>34.999205302839798</v>
+      </c>
+      <c r="E4" s="3">
+        <v>34.071690757266303</v>
+      </c>
+      <c r="F4" s="3">
+        <v>25.513145741921299</v>
+      </c>
+      <c r="G4" s="3">
+        <v>56.043513957307098</v>
+      </c>
+      <c r="H4" s="3">
+        <v>46.330049261083701</v>
+      </c>
+      <c r="I4" s="3">
+        <v>39.755336617405597</v>
+      </c>
+      <c r="J4" s="3">
+        <v>96.275730104300393</v>
+      </c>
+      <c r="K4" s="3">
+        <v>93.597320133511005</v>
+      </c>
+      <c r="L4" s="3">
+        <v>87.007258193659197</v>
+      </c>
+      <c r="M4" s="3">
+        <v>13.5296059082648</v>
+      </c>
+      <c r="N4" s="3">
+        <v>12.042179159048599</v>
+      </c>
+      <c r="O4" s="3">
+        <v>10.3533366648712</v>
+      </c>
+      <c r="P4" s="3">
+        <v>88.084923863196494</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>80.102223186971599</v>
+      </c>
+      <c r="R4" s="3">
+        <v>47.895015168535799</v>
+      </c>
+      <c r="S4" s="3">
+        <v>91.093759071187606</v>
+      </c>
+      <c r="T4" s="3">
+        <v>84.323639727301796</v>
+      </c>
+      <c r="U4" s="3">
+        <v>63.439366686571802</v>
+      </c>
+      <c r="V4" s="3">
+        <v>78.6301607461033</v>
+      </c>
+      <c r="W4" s="3">
+        <v>68.710362517131799</v>
+      </c>
+      <c r="X4" s="3">
+        <v>39.7052682914968</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A5" s="3">
+        <v>23.9903784814251</v>
+      </c>
+      <c r="B5" s="3">
+        <v>23.9903784814251</v>
+      </c>
+      <c r="C5" s="3">
+        <v>23.9903784814251</v>
+      </c>
+      <c r="D5" s="3">
+        <v>14.899698206656501</v>
+      </c>
+      <c r="E5" s="3">
+        <v>14.899698206656501</v>
+      </c>
+      <c r="F5" s="3">
+        <v>14.899698206656501</v>
+      </c>
+      <c r="G5" s="3">
+        <v>55.127652233914098</v>
+      </c>
+      <c r="H5" s="3">
+        <v>55.124719682594403</v>
+      </c>
+      <c r="I5" s="3">
+        <v>55.122304640331201</v>
+      </c>
+      <c r="J5" s="3">
+        <v>92.433866927760107</v>
+      </c>
+      <c r="K5" s="3">
+        <v>92.433866927760107</v>
+      </c>
+      <c r="L5" s="3">
+        <v>92.433866927760107</v>
+      </c>
+      <c r="M5" s="3">
+        <v>7.4626280101308398</v>
+      </c>
+      <c r="N5" s="3">
+        <v>7.4626280101308398</v>
+      </c>
+      <c r="O5" s="3">
+        <v>7.4626280101308398</v>
+      </c>
+      <c r="P5" s="3">
+        <v>92.026591024708395</v>
+      </c>
+      <c r="Q5" s="3">
+        <v>92.026591024708395</v>
+      </c>
+      <c r="R5" s="3">
+        <v>92.026591024708395</v>
+      </c>
+      <c r="S5" s="3">
+        <v>91.451158336004099</v>
+      </c>
+      <c r="T5" s="3">
+        <v>91.441609030873096</v>
+      </c>
+      <c r="U5" s="3">
+        <v>91.441609030873096</v>
+      </c>
+      <c r="V5" s="3">
+        <v>79.030386302093106</v>
+      </c>
+      <c r="W5" s="3">
+        <v>79.030386302093106</v>
+      </c>
+      <c r="X5" s="3">
+        <v>79.030386302093106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A6" s="3">
+        <v>30.480872526915402</v>
+      </c>
+      <c r="B6" s="3">
+        <v>30.480872526915402</v>
+      </c>
+      <c r="C6" s="3">
+        <v>30.480872526915402</v>
+      </c>
+      <c r="D6" s="3">
+        <v>13.696402379602899</v>
+      </c>
+      <c r="E6" s="3">
+        <v>13.696402379602899</v>
+      </c>
+      <c r="F6" s="3">
+        <v>13.696402379602899</v>
+      </c>
+      <c r="G6" s="3">
+        <v>63.206944444444403</v>
+      </c>
+      <c r="H6" s="3">
+        <v>63.206944444444403</v>
+      </c>
+      <c r="I6" s="3">
+        <v>63.206944444444403</v>
+      </c>
+      <c r="J6" s="3">
+        <v>92.651127705379096</v>
+      </c>
+      <c r="K6" s="3">
+        <v>92.651127705379096</v>
+      </c>
+      <c r="L6" s="3">
+        <v>92.651127705379096</v>
+      </c>
+      <c r="M6" s="3">
+        <v>26.3800132374528</v>
+      </c>
+      <c r="N6" s="3">
+        <v>26.3800132374528</v>
+      </c>
+      <c r="O6" s="3">
+        <v>26.3800132374528</v>
+      </c>
+      <c r="P6" s="3">
+        <v>93.691574431161996</v>
+      </c>
+      <c r="Q6" s="3">
+        <v>93.691574431161996</v>
+      </c>
+      <c r="R6" s="3">
+        <v>93.691574431161996</v>
+      </c>
+      <c r="S6" s="3">
+        <v>92.743437187760307</v>
+      </c>
+      <c r="T6" s="3">
+        <v>92.743437187760307</v>
+      </c>
+      <c r="U6" s="3">
+        <v>92.743437187760307</v>
+      </c>
+      <c r="V6" s="3">
+        <v>86.916038226513194</v>
+      </c>
+      <c r="W6" s="3">
+        <v>86.916038226513194</v>
+      </c>
+      <c r="X6" s="3">
+        <v>86.916038226513194</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A7" s="3">
+        <v>18.0519533296088</v>
+      </c>
+      <c r="B7" s="3">
+        <v>15.727314637214899</v>
+      </c>
+      <c r="C7" s="3">
+        <v>8.2788390090075694</v>
+      </c>
+      <c r="D7" s="3">
+        <v>26.8571084099326</v>
+      </c>
+      <c r="E7" s="3">
+        <v>24.955659288932601</v>
+      </c>
+      <c r="F7" s="3">
+        <v>15.099958779863</v>
+      </c>
+      <c r="G7" s="3">
+        <v>54.891099855282199</v>
+      </c>
+      <c r="H7" s="3">
+        <v>44.735166425470297</v>
+      </c>
+      <c r="I7" s="3">
+        <v>38.496020260492003</v>
+      </c>
+      <c r="J7" s="3">
+        <v>96.680226171264707</v>
+      </c>
+      <c r="K7" s="3">
+        <v>94.735931824673997</v>
+      </c>
+      <c r="L7" s="3">
+        <v>88.136837629916798</v>
+      </c>
+      <c r="M7" s="3">
+        <v>8.6885227611932905</v>
+      </c>
+      <c r="N7" s="3">
+        <v>6.9965234761677699</v>
+      </c>
+      <c r="O7" s="3">
+        <v>5.1184096117400202</v>
+      </c>
+      <c r="P7" s="3">
+        <v>85.018172537264306</v>
+      </c>
+      <c r="Q7" s="3">
+        <v>75.635279155419198</v>
+      </c>
+      <c r="R7" s="3">
+        <v>47.926921899596799</v>
+      </c>
+      <c r="S7" s="3">
+        <v>90.689686024033904</v>
+      </c>
+      <c r="T7" s="3">
+        <v>84.157734445850906</v>
+      </c>
+      <c r="U7" s="3">
+        <v>63.659863960960003</v>
+      </c>
+      <c r="V7" s="3">
+        <v>79.239142777099303</v>
+      </c>
+      <c r="W7" s="3">
+        <v>69.895246069921299</v>
+      </c>
+      <c r="X7" s="3">
+        <v>43.770860321629698</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
+        <v>30.488153297890499</v>
+      </c>
+      <c r="B8" s="3">
+        <v>30.488153297890499</v>
+      </c>
+      <c r="C8" s="3">
+        <v>30.472591341769299</v>
+      </c>
+      <c r="D8" s="3">
+        <v>26.851595294241299</v>
+      </c>
+      <c r="E8" s="3">
+        <v>26.851595294241299</v>
+      </c>
+      <c r="F8" s="3">
+        <v>26.836033338124199</v>
+      </c>
+      <c r="G8" s="3">
+        <v>50.664958238420702</v>
+      </c>
+      <c r="H8" s="3">
+        <v>50.6076309794989</v>
+      </c>
+      <c r="I8" s="3">
+        <v>50.567767653758501</v>
+      </c>
+      <c r="J8" s="3">
+        <v>92.024964523856198</v>
+      </c>
+      <c r="K8" s="3">
+        <v>92.024964523856198</v>
+      </c>
+      <c r="L8" s="3">
+        <v>91.999928863320505</v>
+      </c>
+      <c r="M8" s="3">
+        <v>7.81337844949336</v>
+      </c>
+      <c r="N8" s="3">
+        <v>7.81337844949336</v>
+      </c>
+      <c r="O8" s="3">
+        <v>7.81337844949336</v>
+      </c>
+      <c r="P8" s="3">
+        <v>90.562158146758307</v>
+      </c>
+      <c r="Q8" s="3">
+        <v>90.524604662732997</v>
+      </c>
+      <c r="R8" s="3">
+        <v>90.377776174392494</v>
+      </c>
+      <c r="S8" s="3">
+        <v>87.977807365935902</v>
+      </c>
+      <c r="T8" s="3">
+        <v>87.952771705406903</v>
+      </c>
+      <c r="U8" s="3">
+        <v>87.846540811579203</v>
+      </c>
+      <c r="V8" s="3">
+        <v>72.107469073825797</v>
+      </c>
+      <c r="W8" s="3">
+        <v>72.094951243559905</v>
+      </c>
+      <c r="X8" s="3">
+        <v>71.951166858923301</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A9" s="3">
+        <v>29.417522860738099</v>
+      </c>
+      <c r="B9" s="3">
+        <v>28.723289683677098</v>
+      </c>
+      <c r="C9" s="3">
+        <v>25.647682926369001</v>
+      </c>
+      <c r="D9" s="3">
+        <v>13.9796642049825</v>
+      </c>
+      <c r="E9" s="3">
+        <v>13.6986624197392</v>
+      </c>
+      <c r="F9" s="3">
+        <v>12.115930170989699</v>
+      </c>
+      <c r="G9" s="3">
+        <v>64.908809891808303</v>
+      </c>
+      <c r="H9" s="3">
+        <v>62.377125193199397</v>
+      </c>
+      <c r="I9" s="3">
+        <v>60.345595054095803</v>
+      </c>
+      <c r="J9" s="3">
+        <v>94.344930263573104</v>
+      </c>
+      <c r="K9" s="3">
+        <v>93.677247430399007</v>
+      </c>
+      <c r="L9" s="3">
+        <v>92.301087025096095</v>
+      </c>
+      <c r="M9" s="3">
+        <v>11.5877848856518</v>
+      </c>
+      <c r="N9" s="3">
+        <v>11.007679100140299</v>
+      </c>
+      <c r="O9" s="3">
+        <v>10.4046081429337</v>
+      </c>
+      <c r="P9" s="3">
+        <v>94.439357331565105</v>
+      </c>
+      <c r="Q9" s="3">
+        <v>93.121718587636494</v>
+      </c>
+      <c r="R9" s="3">
+        <v>86.266658159955696</v>
+      </c>
+      <c r="S9" s="3">
+        <v>92.733934530779294</v>
+      </c>
+      <c r="T9" s="3">
+        <v>91.561534587752305</v>
+      </c>
+      <c r="U9" s="3">
+        <v>87.848758030687407</v>
+      </c>
+      <c r="V9" s="3">
+        <v>90.461782783595197</v>
+      </c>
+      <c r="W9" s="3">
+        <v>89.142198940954898</v>
+      </c>
+      <c r="X9" s="3">
+        <v>82.395616449508196</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
+        <v>36.589333896154002</v>
+      </c>
+      <c r="B10" s="3">
+        <v>36.589333896154002</v>
+      </c>
+      <c r="C10" s="3">
+        <v>36.589333896154002</v>
+      </c>
+      <c r="D10" s="3">
+        <v>36.948103825778702</v>
+      </c>
+      <c r="E10" s="3">
+        <v>36.948103825778702</v>
+      </c>
+      <c r="F10" s="3">
+        <v>36.948103825778702</v>
+      </c>
+      <c r="G10" s="3">
+        <v>34.585158150851598</v>
+      </c>
+      <c r="H10" s="3">
+        <v>34.583105231143499</v>
+      </c>
+      <c r="I10" s="3">
+        <v>34.5821928223844</v>
+      </c>
+      <c r="J10" s="3">
+        <v>98.108100149797707</v>
+      </c>
+      <c r="K10" s="3">
+        <v>98.108100149797707</v>
+      </c>
+      <c r="L10" s="3">
+        <v>98.100093754055393</v>
+      </c>
+      <c r="M10" s="3">
+        <v>9.5459134721647398</v>
+      </c>
+      <c r="N10" s="3">
+        <v>9.5459134721647398</v>
+      </c>
+      <c r="O10" s="3">
+        <v>9.5459134721647398</v>
+      </c>
+      <c r="P10" s="3">
+        <v>86.357557707755205</v>
+      </c>
+      <c r="Q10" s="3">
+        <v>86.357557707755205</v>
+      </c>
+      <c r="R10" s="3">
+        <v>86.357557707755205</v>
+      </c>
+      <c r="S10" s="3">
+        <v>85.268111219979801</v>
+      </c>
+      <c r="T10" s="3">
+        <v>85.260104823150996</v>
+      </c>
+      <c r="U10" s="3">
+        <v>85.260104823150996</v>
+      </c>
+      <c r="V10" s="3">
+        <v>47.6739396747585</v>
+      </c>
+      <c r="W10" s="3">
+        <v>47.6739396747585</v>
+      </c>
+      <c r="X10" s="3">
+        <v>47.6739396747585</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A11" s="3">
+        <v>42.824769906492499</v>
+      </c>
+      <c r="B11" s="3">
+        <v>37.8685150073103</v>
+      </c>
+      <c r="C11" s="3">
+        <v>12.8678503304321</v>
+      </c>
+      <c r="D11" s="3">
+        <v>47.288167317442898</v>
+      </c>
+      <c r="E11" s="3">
+        <v>45.024047213144698</v>
+      </c>
+      <c r="F11" s="3">
+        <v>24.499434316546498</v>
+      </c>
+      <c r="G11" s="3">
+        <v>59.967086765241</v>
+      </c>
+      <c r="H11" s="3">
+        <v>45.998081439581902</v>
+      </c>
+      <c r="I11" s="3">
+        <v>36.855810260990403</v>
+      </c>
+      <c r="J11" s="3">
+        <v>98.629945625159607</v>
+      </c>
+      <c r="K11" s="3">
+        <v>97.622002750885002</v>
+      </c>
+      <c r="L11" s="3">
+        <v>92.171590485496793</v>
+      </c>
+      <c r="M11" s="3">
+        <v>7.4369118015606199</v>
+      </c>
+      <c r="N11" s="3">
+        <v>4.7130132513206897</v>
+      </c>
+      <c r="O11" s="3">
+        <v>2.5892856413293099</v>
+      </c>
+      <c r="P11" s="3">
+        <v>84.401088752188002</v>
+      </c>
+      <c r="Q11" s="3">
+        <v>71.624162645318293</v>
+      </c>
+      <c r="R11" s="3">
+        <v>38.487705291512199</v>
+      </c>
+      <c r="S11" s="3">
+        <v>92.951306307618594</v>
+      </c>
+      <c r="T11" s="3">
+        <v>85.611855051948197</v>
+      </c>
+      <c r="U11" s="3">
+        <v>60.744090984076699</v>
+      </c>
+      <c r="V11" s="3">
+        <v>81.062091851484993</v>
+      </c>
+      <c r="W11" s="3">
+        <v>69.809704843527101</v>
+      </c>
+      <c r="X11" s="3">
+        <v>35.530885278765801</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
+        <v>35.023951334694502</v>
+      </c>
+      <c r="B12" s="3">
+        <v>29.116316831975499</v>
+      </c>
+      <c r="C12" s="3">
+        <v>10.1807462705743</v>
+      </c>
+      <c r="D12" s="3">
+        <v>31.374218697846601</v>
+      </c>
+      <c r="E12" s="3">
+        <v>27.397786215381299</v>
+      </c>
+      <c r="F12" s="3">
+        <v>10.514210073979701</v>
+      </c>
+      <c r="G12" s="3">
+        <v>52.165337833905603</v>
+      </c>
+      <c r="H12" s="3">
+        <v>34.244951405458899</v>
+      </c>
+      <c r="I12" s="3">
+        <v>25.475877320607601</v>
+      </c>
+      <c r="J12" s="3">
+        <v>98.835112551632506</v>
+      </c>
+      <c r="K12" s="3">
+        <v>96.359790620350296</v>
+      </c>
+      <c r="L12" s="3">
+        <v>80.451096417885296</v>
+      </c>
+      <c r="M12" s="3">
+        <v>9.5711616024735502</v>
+      </c>
+      <c r="N12" s="3">
+        <v>5.4891980275718</v>
+      </c>
+      <c r="O12" s="3">
+        <v>2.6768233253868101</v>
+      </c>
+      <c r="P12" s="3">
+        <v>64.138992199606804</v>
+      </c>
+      <c r="Q12" s="3">
+        <v>46.187863083281499</v>
+      </c>
+      <c r="R12" s="3">
+        <v>21.7287280033899</v>
+      </c>
+      <c r="S12" s="3">
+        <v>82.703785410237899</v>
+      </c>
+      <c r="T12" s="3">
+        <v>64.7203914733293</v>
+      </c>
+      <c r="U12" s="3">
+        <v>37.346959563214099</v>
+      </c>
+      <c r="V12" s="3">
+        <v>68.812070671374798</v>
+      </c>
+      <c r="W12" s="3">
+        <v>52.449962747489501</v>
+      </c>
+      <c r="X12" s="3">
+        <v>24.763810918890801</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>45.108726634025302</v>
+      </c>
+      <c r="B13" s="3">
+        <v>38.392851577977297</v>
+      </c>
+      <c r="C13" s="3">
+        <v>15.521351330897</v>
+      </c>
+      <c r="D13" s="3">
+        <v>7.8978610827940603</v>
+      </c>
+      <c r="E13" s="3">
+        <v>6.9027937923159604</v>
+      </c>
+      <c r="F13" s="3">
+        <v>3.6543897997980501</v>
+      </c>
+      <c r="G13" s="3">
+        <v>82.399343031440594</v>
+      </c>
+      <c r="H13" s="3">
+        <v>61.000938526513401</v>
+      </c>
+      <c r="I13" s="3">
+        <v>43.089629282027197</v>
+      </c>
+      <c r="J13" s="3">
+        <v>96.980162316401106</v>
+      </c>
+      <c r="K13" s="3">
+        <v>93.574711850306002</v>
+      </c>
+      <c r="L13" s="3">
+        <v>69.265307871383996</v>
+      </c>
+      <c r="M13" s="3">
+        <v>51.916550175123099</v>
+      </c>
+      <c r="N13" s="3">
+        <v>32.308462401458499</v>
+      </c>
+      <c r="O13" s="3">
+        <v>18.1730722143332</v>
+      </c>
+      <c r="P13" s="3">
+        <v>86.170316485844097</v>
+      </c>
+      <c r="Q13" s="3">
+        <v>70.194175351561498</v>
+      </c>
+      <c r="R13" s="3">
+        <v>32.877515882188298</v>
+      </c>
+      <c r="S13" s="3">
+        <v>90.891037427155695</v>
+      </c>
+      <c r="T13" s="3">
+        <v>82.097542326475505</v>
+      </c>
+      <c r="U13" s="3">
+        <v>41.532323047951401</v>
+      </c>
+      <c r="V13" s="3">
+        <v>94.149302385300899</v>
+      </c>
+      <c r="W13" s="3">
+        <v>88.039938028590697</v>
+      </c>
+      <c r="X13" s="3">
+        <v>36.8878743494666</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A14" s="3">
+        <v>67.942329839569098</v>
+      </c>
+      <c r="B14" s="3">
+        <v>62.324103047434498</v>
+      </c>
+      <c r="C14" s="3">
+        <v>29.741732357401801</v>
+      </c>
+      <c r="D14" s="3">
+        <v>60.1332354297382</v>
+      </c>
+      <c r="E14" s="3">
+        <v>56.742662524985001</v>
+      </c>
+      <c r="F14" s="3">
+        <v>27.868177144400502</v>
+      </c>
+      <c r="G14" s="3">
+        <v>89.987565282268093</v>
+      </c>
+      <c r="H14" s="3">
+        <v>73.594130813230507</v>
+      </c>
+      <c r="I14" s="3">
+        <v>57.435961203680698</v>
+      </c>
+      <c r="J14" s="3">
+        <v>96.594488667522597</v>
+      </c>
+      <c r="K14" s="3">
+        <v>90.384060413119499</v>
+      </c>
+      <c r="L14" s="3">
+        <v>70.570843281477394</v>
+      </c>
+      <c r="M14" s="3">
+        <v>80.733401639219096</v>
+      </c>
+      <c r="N14" s="3">
+        <v>65.806573119574097</v>
+      </c>
+      <c r="O14" s="3">
+        <v>35.642626615605899</v>
+      </c>
+      <c r="P14" s="3">
+        <v>81.042050851866094</v>
+      </c>
+      <c r="Q14" s="3">
+        <v>66.265381716532005</v>
+      </c>
+      <c r="R14" s="3">
+        <v>35.7115054509812</v>
+      </c>
+      <c r="S14" s="3">
+        <v>93.108421002306301</v>
+      </c>
+      <c r="T14" s="3">
+        <v>85.059650066061096</v>
+      </c>
+      <c r="U14" s="3">
+        <v>56.071106602789001</v>
+      </c>
+      <c r="V14" s="3">
+        <v>95.466848726447594</v>
+      </c>
+      <c r="W14" s="3">
+        <v>89.891840053292398</v>
+      </c>
+      <c r="X14" s="3">
+        <v>47.695158363979601</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A15" s="3">
+        <v>74.4191271935548</v>
+      </c>
+      <c r="B15" s="3">
+        <v>69.149655775703707</v>
+      </c>
+      <c r="C15" s="3">
+        <v>22.869268221422601</v>
+      </c>
+      <c r="D15" s="3">
+        <v>61.569383898875998</v>
+      </c>
+      <c r="E15" s="3">
+        <v>57.208121355037697</v>
+      </c>
+      <c r="F15" s="3">
+        <v>25.514928408850501</v>
+      </c>
+      <c r="G15" s="3">
+        <v>95.813658536585393</v>
+      </c>
+      <c r="H15" s="3">
+        <v>76.727154471544694</v>
+      </c>
+      <c r="I15" s="3">
+        <v>54.853658536585399</v>
+      </c>
+      <c r="J15" s="3">
+        <v>96.469832011789805</v>
+      </c>
+      <c r="K15" s="3">
+        <v>89.072052374142899</v>
+      </c>
+      <c r="L15" s="3">
+        <v>67.033351686821007</v>
+      </c>
+      <c r="M15" s="3">
+        <v>86.909743511315099</v>
+      </c>
+      <c r="N15" s="3">
+        <v>66.361144670880194</v>
+      </c>
+      <c r="O15" s="3">
+        <v>27.931353740620501</v>
+      </c>
+      <c r="P15" s="3">
+        <v>75.9819404443422</v>
+      </c>
+      <c r="Q15" s="3">
+        <v>55.539306721265099</v>
+      </c>
+      <c r="R15" s="3">
+        <v>24.520145867394199</v>
+      </c>
+      <c r="S15" s="3">
+        <v>95.975629996066601</v>
+      </c>
+      <c r="T15" s="3">
+        <v>83.080704082700805</v>
+      </c>
+      <c r="U15" s="3">
+        <v>46.773403010746101</v>
+      </c>
+      <c r="V15" s="3">
+        <v>98.713022673795393</v>
+      </c>
+      <c r="W15" s="3">
+        <v>91.951988792614401</v>
+      </c>
+      <c r="X15" s="3">
+        <v>38.090419866474697</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A16" s="3">
+        <v>83.888097020798497</v>
+      </c>
+      <c r="B16" s="3">
+        <v>79.280496594592606</v>
+      </c>
+      <c r="C16" s="3">
+        <v>21.983207360121099</v>
+      </c>
+      <c r="D16" s="3">
+        <v>73.054889558095994</v>
+      </c>
+      <c r="E16" s="3">
+        <v>68.811906816229396</v>
+      </c>
+      <c r="F16" s="3">
+        <v>27.319747747266099</v>
+      </c>
+      <c r="G16" s="3">
+        <v>97.025311203319504</v>
+      </c>
+      <c r="H16" s="3">
+        <v>77.750829875518704</v>
+      </c>
+      <c r="I16" s="3">
+        <v>53.4836099585062</v>
+      </c>
+      <c r="J16" s="3">
+        <v>99.092716590605605</v>
+      </c>
+      <c r="K16" s="3">
+        <v>96.505938348835599</v>
+      </c>
+      <c r="L16" s="3">
+        <v>80.333410768622997</v>
+      </c>
+      <c r="M16" s="3">
+        <v>93.933707686176206</v>
+      </c>
+      <c r="N16" s="3">
+        <v>75.444458665729201</v>
+      </c>
+      <c r="O16" s="3">
+        <v>27.230814124292699</v>
+      </c>
+      <c r="P16" s="3">
+        <v>86.972455113439594</v>
+      </c>
+      <c r="Q16" s="3">
+        <v>65.419411872601501</v>
+      </c>
+      <c r="R16" s="3">
+        <v>23.382128582588901</v>
+      </c>
+      <c r="S16" s="3">
+        <v>99.364479620802499</v>
+      </c>
+      <c r="T16" s="3">
+        <v>94.202752355415399</v>
+      </c>
+      <c r="U16" s="3">
+        <v>52.539836792085602</v>
+      </c>
+      <c r="V16" s="3">
+        <v>99.732253181022003</v>
+      </c>
+      <c r="W16" s="3">
+        <v>96.337414355603798</v>
+      </c>
+      <c r="X16" s="3">
+        <v>34.698657265820202</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A17" s="3">
+        <v>81.495878856592697</v>
+      </c>
+      <c r="B17" s="3">
+        <v>70.584896500320397</v>
+      </c>
+      <c r="C17" s="3">
+        <v>7.4573378515157804</v>
+      </c>
+      <c r="D17" s="3">
+        <v>68.795044501762007</v>
+      </c>
+      <c r="E17" s="3">
+        <v>59.750399728601501</v>
+      </c>
+      <c r="F17" s="3">
+        <v>7.7690994082225604</v>
+      </c>
+      <c r="G17" s="3">
+        <v>95.069799777530605</v>
+      </c>
+      <c r="H17" s="3">
+        <v>51.511123470522797</v>
+      </c>
+      <c r="I17" s="3">
+        <v>22.062291434927701</v>
+      </c>
+      <c r="J17" s="3">
+        <v>97.784730376320596</v>
+      </c>
+      <c r="K17" s="3">
+        <v>79.544698300218201</v>
+      </c>
+      <c r="L17" s="3">
+        <v>22.590915235405699</v>
+      </c>
+      <c r="M17" s="3">
+        <v>94.335865944532102</v>
+      </c>
+      <c r="N17" s="3">
+        <v>50.718640368690799</v>
+      </c>
+      <c r="O17" s="3">
+        <v>9.0711673224858593</v>
+      </c>
+      <c r="P17" s="3">
+        <v>89.957045171184006</v>
+      </c>
+      <c r="Q17" s="3">
+        <v>47.4164768536317</v>
+      </c>
+      <c r="R17" s="3">
+        <v>8.5586382921671493</v>
+      </c>
+      <c r="S17" s="3">
+        <v>98.6023306325405</v>
+      </c>
+      <c r="T17" s="3">
+        <v>78.359386203238998</v>
+      </c>
+      <c r="U17" s="3">
+        <v>15.5677149931828</v>
+      </c>
+      <c r="V17" s="3">
+        <v>99.377670799270206</v>
+      </c>
+      <c r="W17" s="3">
+        <v>89.578711960969002</v>
+      </c>
+      <c r="X17" s="3">
+        <v>11.7242933692908</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A18" s="3">
+        <v>54.184976237581502</v>
+      </c>
+      <c r="B18" s="3">
+        <v>42.296576657951498</v>
+      </c>
+      <c r="C18" s="3">
+        <v>4.7139987024897101</v>
+      </c>
+      <c r="D18" s="3">
+        <v>44.694170182338198</v>
+      </c>
+      <c r="E18" s="3">
+        <v>37.707121433132002</v>
+      </c>
+      <c r="F18" s="3">
+        <v>4.4808428170733698</v>
+      </c>
+      <c r="G18" s="3">
+        <v>81.835324571883703</v>
+      </c>
+      <c r="H18" s="3">
+        <v>41.584229390681003</v>
+      </c>
+      <c r="I18" s="3">
+        <v>20.6919553962565</v>
+      </c>
+      <c r="J18" s="3">
+        <v>98.034883886606593</v>
+      </c>
+      <c r="K18" s="3">
+        <v>88.352224282091299</v>
+      </c>
+      <c r="L18" s="3">
+        <v>47.616511289925299</v>
+      </c>
+      <c r="M18" s="3">
+        <v>78.946620894472503</v>
+      </c>
+      <c r="N18" s="3">
+        <v>37.845059308953402</v>
+      </c>
+      <c r="O18" s="3">
+        <v>6.5747567939707396</v>
+      </c>
+      <c r="P18" s="3">
+        <v>77.487907835615502</v>
+      </c>
+      <c r="Q18" s="3">
+        <v>35.642963897348999</v>
+      </c>
+      <c r="R18" s="3">
+        <v>6.8565107857237102</v>
+      </c>
+      <c r="S18" s="3">
+        <v>94.166356763257198</v>
+      </c>
+      <c r="T18" s="3">
+        <v>67.992657443869106</v>
+      </c>
+      <c r="U18" s="3">
+        <v>12.7682891959789</v>
+      </c>
+      <c r="V18" s="3">
+        <v>96.946389165887396</v>
+      </c>
+      <c r="W18" s="3">
+        <v>79.292059112938801</v>
+      </c>
+      <c r="X18" s="3">
+        <v>8.7395783700028602</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A19" s="3">
+        <v>69.685616582645096</v>
+      </c>
+      <c r="B19" s="3">
+        <v>64.049066599284203</v>
+      </c>
+      <c r="C19" s="3">
+        <v>25.882033234137701</v>
+      </c>
+      <c r="D19" s="3">
+        <v>69.635407994800602</v>
+      </c>
+      <c r="E19" s="3">
+        <v>65.882400091303197</v>
+      </c>
+      <c r="F19" s="3">
+        <v>26.174773849426099</v>
+      </c>
+      <c r="G19" s="3">
+        <v>94.254126440361304</v>
+      </c>
+      <c r="H19" s="3">
+        <v>75.481469947056993</v>
+      </c>
+      <c r="I19" s="3">
+        <v>54.898785425101202</v>
+      </c>
+      <c r="J19" s="3">
+        <v>96.695612897051603</v>
+      </c>
+      <c r="K19" s="3">
+        <v>88.680565315328096</v>
+      </c>
+      <c r="L19" s="3">
+        <v>60.656044602245103</v>
+      </c>
+      <c r="M19" s="3">
+        <v>90.452534179985193</v>
+      </c>
+      <c r="N19" s="3">
+        <v>72.9965642741561</v>
+      </c>
+      <c r="O19" s="3">
+        <v>34.527873249309998</v>
+      </c>
+      <c r="P19" s="3">
+        <v>92.534970765062894</v>
+      </c>
+      <c r="Q19" s="3">
+        <v>73.576783643262402</v>
+      </c>
+      <c r="R19" s="3">
+        <v>34.8291961853526</v>
+      </c>
+      <c r="S19" s="3">
+        <v>98.693898336996</v>
+      </c>
+      <c r="T19" s="3">
+        <v>90.747439282692795</v>
+      </c>
+      <c r="U19" s="3">
+        <v>53.451027419732803</v>
+      </c>
+      <c r="V19" s="3">
+        <v>99.559652087063299</v>
+      </c>
+      <c r="W19" s="3">
+        <v>95.599933495300206</v>
+      </c>
+      <c r="X19" s="3">
+        <v>41.3567514915594</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A20" s="3">
+        <v>77.056591975510699</v>
+      </c>
+      <c r="B20" s="3">
+        <v>70.281215103774002</v>
+      </c>
+      <c r="C20" s="3">
+        <v>19.132155334199201</v>
+      </c>
+      <c r="D20" s="3">
+        <v>62.203817835774899</v>
+      </c>
+      <c r="E20" s="3">
+        <v>57.1292521962528</v>
+      </c>
+      <c r="F20" s="3">
+        <v>20.3802880560368</v>
+      </c>
+      <c r="G20" s="3">
+        <v>91.562456058120503</v>
+      </c>
+      <c r="H20" s="3">
+        <v>70.584251230372601</v>
+      </c>
+      <c r="I20" s="3">
+        <v>49.114366065151202</v>
+      </c>
+      <c r="J20" s="3">
+        <v>98.311261867056402</v>
+      </c>
+      <c r="K20" s="3">
+        <v>95.456528330165796</v>
+      </c>
+      <c r="L20" s="3">
+        <v>78.223091899647798</v>
+      </c>
+      <c r="M20" s="3">
+        <v>89.254921254609897</v>
+      </c>
+      <c r="N20" s="3">
+        <v>70.061729804364603</v>
+      </c>
+      <c r="O20" s="3">
+        <v>24.9961523506981</v>
+      </c>
+      <c r="P20" s="3">
+        <v>91.266762166223899</v>
+      </c>
+      <c r="Q20" s="3">
+        <v>75.018113049059295</v>
+      </c>
+      <c r="R20" s="3">
+        <v>26.2003331477088</v>
+      </c>
+      <c r="S20" s="3">
+        <v>98.596959724942195</v>
+      </c>
+      <c r="T20" s="3">
+        <v>93.148741465465307</v>
+      </c>
+      <c r="U20" s="3">
+        <v>50.796836605122998</v>
+      </c>
+      <c r="V20" s="3">
+        <v>99.099105785024307</v>
+      </c>
+      <c r="W20" s="3">
+        <v>96.039374305375603</v>
+      </c>
+      <c r="X20" s="3">
+        <v>34.1546871272066</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A21" s="3">
+        <v>58.559846869254201</v>
+      </c>
+      <c r="B21" s="3">
+        <v>50.680001847172903</v>
+      </c>
+      <c r="C21" s="3">
+        <v>8.8128470568208304</v>
+      </c>
+      <c r="D21" s="3">
+        <v>54.386963366027302</v>
+      </c>
+      <c r="E21" s="3">
+        <v>50.167212564351601</v>
+      </c>
+      <c r="F21" s="3">
+        <v>16.834330826129801</v>
+      </c>
+      <c r="G21" s="3">
+        <v>76.997792372647496</v>
+      </c>
+      <c r="H21" s="3">
+        <v>52.377449086594197</v>
+      </c>
+      <c r="I21" s="3">
+        <v>35.772007285170297</v>
+      </c>
+      <c r="J21" s="3">
+        <v>97.597878901472399</v>
+      </c>
+      <c r="K21" s="3">
+        <v>92.703235521430898</v>
+      </c>
+      <c r="L21" s="3">
+        <v>70.613910866457701</v>
+      </c>
+      <c r="M21" s="3">
+        <v>56.437898798593203</v>
+      </c>
+      <c r="N21" s="3">
+        <v>34.682890076523897</v>
+      </c>
+      <c r="O21" s="3">
+        <v>10.7664364376039</v>
+      </c>
+      <c r="P21" s="3">
+        <v>81.052521457330499</v>
+      </c>
+      <c r="Q21" s="3">
+        <v>58.010112387126703</v>
+      </c>
+      <c r="R21" s="3">
+        <v>16.784721611460899</v>
+      </c>
+      <c r="S21" s="3">
+        <v>95.587045940787306</v>
+      </c>
+      <c r="T21" s="3">
+        <v>84.657888147045199</v>
+      </c>
+      <c r="U21" s="3">
+        <v>44.518697087451599</v>
+      </c>
+      <c r="V21" s="3">
+        <v>94.653847911116102</v>
+      </c>
+      <c r="W21" s="3">
+        <v>82.993890643857597</v>
+      </c>
+      <c r="X21" s="3">
+        <v>26.835371387758499</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A22" s="3">
+        <v>59.847300879612803</v>
+      </c>
+      <c r="B22" s="3">
+        <v>53.628767709195003</v>
+      </c>
+      <c r="C22" s="3">
+        <v>14.232247362893</v>
+      </c>
+      <c r="D22" s="3">
+        <v>69.022323752085001</v>
+      </c>
+      <c r="E22" s="3">
+        <v>66.435287526898193</v>
+      </c>
+      <c r="F22" s="3">
+        <v>35.338378372204701</v>
+      </c>
+      <c r="G22" s="3">
+        <v>71.924780150753804</v>
+      </c>
+      <c r="H22" s="3">
+        <v>52.816739949748701</v>
+      </c>
+      <c r="I22" s="3">
+        <v>39.094221105527602</v>
+      </c>
+      <c r="J22" s="3">
+        <v>99.042795791699803</v>
+      </c>
+      <c r="K22" s="3">
+        <v>97.129632854824706</v>
+      </c>
+      <c r="L22" s="3">
+        <v>86.155366070668606</v>
+      </c>
+      <c r="M22" s="3">
+        <v>40.571425320370203</v>
+      </c>
+      <c r="N22" s="3">
+        <v>27.061606820234999</v>
+      </c>
+      <c r="O22" s="3">
+        <v>10.2016849062886</v>
+      </c>
+      <c r="P22" s="3">
+        <v>80.541867777525198</v>
+      </c>
+      <c r="Q22" s="3">
+        <v>63.9962146415223</v>
+      </c>
+      <c r="R22" s="3">
+        <v>25.238283734166401</v>
+      </c>
+      <c r="S22" s="3">
+        <v>93.819621748318099</v>
+      </c>
+      <c r="T22" s="3">
+        <v>85.439504257001104</v>
+      </c>
+      <c r="U22" s="3">
+        <v>53.858570992498599</v>
+      </c>
+      <c r="V22" s="3">
+        <v>87.716424503120706</v>
+      </c>
+      <c r="W22" s="3">
+        <v>77.942927274254203</v>
+      </c>
+      <c r="X22" s="3">
+        <v>31.508368559121699</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A23" s="3">
+        <v>59.062063896912001</v>
+      </c>
+      <c r="B23" s="3">
+        <v>49.762454550390103</v>
+      </c>
+      <c r="C23" s="3">
+        <v>10.0315779031642</v>
+      </c>
+      <c r="D23" s="3">
+        <v>83.934729419021707</v>
+      </c>
+      <c r="E23" s="3">
+        <v>81.589309078858093</v>
+      </c>
+      <c r="F23" s="3">
+        <v>32.425289710519699</v>
+      </c>
+      <c r="G23" s="3">
+        <v>83.530129755882996</v>
+      </c>
+      <c r="H23" s="3">
+        <v>53.981306355839003</v>
+      </c>
+      <c r="I23" s="3">
+        <v>34.016714317132198</v>
+      </c>
+      <c r="J23" s="3">
+        <v>98.012536198007695</v>
+      </c>
+      <c r="K23" s="3">
+        <v>92.172911836720104</v>
+      </c>
+      <c r="L23" s="3">
+        <v>69.104437665907199</v>
+      </c>
+      <c r="M23" s="3">
+        <v>69.825045647306197</v>
+      </c>
+      <c r="N23" s="3">
+        <v>41.113309654547997</v>
+      </c>
+      <c r="O23" s="3">
+        <v>12.3686514710125</v>
+      </c>
+      <c r="P23" s="3">
+        <v>81.880184651979306</v>
+      </c>
+      <c r="Q23" s="3">
+        <v>57.550984617984298</v>
+      </c>
+      <c r="R23" s="3">
+        <v>17.763362212683901</v>
+      </c>
+      <c r="S23" s="3">
+        <v>96.801430949573799</v>
+      </c>
+      <c r="T23" s="3">
+        <v>85.513063499906295</v>
+      </c>
+      <c r="U23" s="3">
+        <v>34.1073740521663</v>
+      </c>
+      <c r="V23" s="3">
+        <v>96.340780893302295</v>
+      </c>
+      <c r="W23" s="3">
+        <v>84.763030829472299</v>
+      </c>
+      <c r="X23" s="3">
+        <v>21.015161070993798</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A24" s="3">
+        <v>49.735156015734503</v>
+      </c>
+      <c r="B24" s="3">
+        <v>39.216345548595001</v>
+      </c>
+      <c r="C24" s="3">
+        <v>8.1877821342145705</v>
+      </c>
+      <c r="D24" s="3">
+        <v>86.096562700670006</v>
+      </c>
+      <c r="E24" s="3">
+        <v>83.143556746302707</v>
+      </c>
+      <c r="F24" s="3">
+        <v>18.094096671703301</v>
+      </c>
+      <c r="G24" s="3">
+        <v>81.217058941862803</v>
+      </c>
+      <c r="H24" s="3">
+        <v>41.197344598672302</v>
+      </c>
+      <c r="I24" s="3">
+        <v>24.594648963991101</v>
+      </c>
+      <c r="J24" s="3">
+        <v>97.613677332326205</v>
+      </c>
+      <c r="K24" s="3">
+        <v>81.912427151408096</v>
+      </c>
+      <c r="L24" s="3">
+        <v>31.939297270117098</v>
+      </c>
+      <c r="M24" s="3">
+        <v>68.495382329566993</v>
+      </c>
+      <c r="N24" s="3">
+        <v>32.527983485187498</v>
+      </c>
+      <c r="O24" s="3">
+        <v>11.7138112748358</v>
+      </c>
+      <c r="P24" s="3">
+        <v>88.684123130744197</v>
+      </c>
+      <c r="Q24" s="3">
+        <v>49.1078302462222</v>
+      </c>
+      <c r="R24" s="3">
+        <v>16.900239935425802</v>
+      </c>
+      <c r="S24" s="3">
+        <v>96.895843732844099</v>
+      </c>
+      <c r="T24" s="3">
+        <v>73.423956168583999</v>
+      </c>
+      <c r="U24" s="3">
+        <v>22.4149815284729</v>
+      </c>
+      <c r="V24" s="3">
+        <v>96.812911635412206</v>
+      </c>
+      <c r="W24" s="3">
+        <v>76.095584531518895</v>
+      </c>
+      <c r="X24" s="3">
+        <v>18.3567059464342</v>
+      </c>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A25" s="3">
+        <v>30.5635144364702</v>
+      </c>
+      <c r="B25" s="3">
+        <v>27.642765589618801</v>
+      </c>
+      <c r="C25" s="3">
+        <v>13.3050801507356</v>
+      </c>
+      <c r="D25" s="3">
+        <v>55.602550253580802</v>
+      </c>
+      <c r="E25" s="3">
+        <v>54.317785748636403</v>
+      </c>
+      <c r="F25" s="3">
+        <v>37.835595668939</v>
+      </c>
+      <c r="G25" s="3">
+        <v>48.174484317603799</v>
+      </c>
+      <c r="H25" s="3">
+        <v>39.833568804747102</v>
+      </c>
+      <c r="I25" s="3">
+        <v>34.643331449561998</v>
+      </c>
+      <c r="J25" s="3">
+        <v>98.394011126883498</v>
+      </c>
+      <c r="K25" s="3">
+        <v>97.370393316914999</v>
+      </c>
+      <c r="L25" s="3">
+        <v>91.452177142652303</v>
+      </c>
+      <c r="M25" s="3">
+        <v>7.3029215668763099</v>
+      </c>
+      <c r="N25" s="3">
+        <v>5.4343075637800897</v>
+      </c>
+      <c r="O25" s="3">
+        <v>3.5992670438023402</v>
+      </c>
+      <c r="P25" s="3">
+        <v>86.519182255574705</v>
+      </c>
+      <c r="Q25" s="3">
+        <v>76.830738117497305</v>
+      </c>
+      <c r="R25" s="3">
+        <v>52.5645535200184</v>
+      </c>
+      <c r="S25" s="3">
+        <v>92.460332094001998</v>
+      </c>
+      <c r="T25" s="3">
+        <v>86.078849799596</v>
+      </c>
+      <c r="U25" s="3">
+        <v>68.461017237797904</v>
+      </c>
+      <c r="V25" s="3">
+        <v>73.488105369355694</v>
+      </c>
+      <c r="W25" s="3">
+        <v>64.019541884112698</v>
+      </c>
+      <c r="X25" s="3">
+        <v>40.286698895045198</v>
+      </c>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A26" s="3">
+        <v>38.150452170686997</v>
+      </c>
+      <c r="B26" s="3">
+        <v>36.062727207076499</v>
+      </c>
+      <c r="C26" s="3">
+        <v>23.836787909665599</v>
+      </c>
+      <c r="D26" s="3">
+        <v>43.448117830764701</v>
+      </c>
+      <c r="E26" s="3">
+        <v>42.1042930963483</v>
+      </c>
+      <c r="F26" s="3">
+        <v>30.286923149854601</v>
+      </c>
+      <c r="G26" s="3">
+        <v>58.972377653432801</v>
+      </c>
+      <c r="H26" s="3">
+        <v>51.872724042987798</v>
+      </c>
+      <c r="I26" s="3">
+        <v>46.716671107558398</v>
+      </c>
+      <c r="J26" s="3">
+        <v>97.968811404335099</v>
+      </c>
+      <c r="K26" s="3">
+        <v>97.372247335260994</v>
+      </c>
+      <c r="L26" s="3">
+        <v>95.003520063445293</v>
+      </c>
+      <c r="M26" s="3">
+        <v>15.726269937040801</v>
+      </c>
+      <c r="N26" s="3">
+        <v>12.889743944056301</v>
+      </c>
+      <c r="O26" s="3">
+        <v>9.2458774151543697</v>
+      </c>
+      <c r="P26" s="3">
+        <v>94.193140545189706</v>
+      </c>
+      <c r="Q26" s="3">
+        <v>90.3098992576315</v>
+      </c>
+      <c r="R26" s="3">
+        <v>72.341823006288905</v>
+      </c>
+      <c r="S26" s="3">
+        <v>94.078978259273399</v>
+      </c>
+      <c r="T26" s="3">
+        <v>91.466219254945401</v>
+      </c>
+      <c r="U26" s="3">
+        <v>79.964306198321694</v>
+      </c>
+      <c r="V26" s="3">
+        <v>87.863685627784704</v>
+      </c>
+      <c r="W26" s="3">
+        <v>84.117569579591802</v>
+      </c>
+      <c r="X26" s="3">
+        <v>65.676437503346804</v>
+      </c>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A27" s="3">
+        <v>34.232747334843097</v>
+      </c>
+      <c r="B27" s="3">
+        <v>32.909852350094503</v>
+      </c>
+      <c r="C27" s="3">
+        <v>25.028486512461601</v>
+      </c>
+      <c r="D27" s="3">
+        <v>44.292158257756</v>
+      </c>
+      <c r="E27" s="3">
+        <v>43.539350572765599</v>
+      </c>
+      <c r="F27" s="3">
+        <v>37.782996846263501</v>
+      </c>
+      <c r="G27" s="3">
+        <v>68.483630952380906</v>
+      </c>
+      <c r="H27" s="3">
+        <v>61.293154761904802</v>
+      </c>
+      <c r="I27" s="3">
+        <v>54.763392857142897</v>
+      </c>
+      <c r="J27" s="3">
+        <v>98.646288968526505</v>
+      </c>
+      <c r="K27" s="3">
+        <v>98.646288968526505</v>
+      </c>
+      <c r="L27" s="3">
+        <v>97.0874122019937</v>
+      </c>
+      <c r="M27" s="3">
+        <v>20.546546776758898</v>
+      </c>
+      <c r="N27" s="3">
+        <v>17.449914996373199</v>
+      </c>
+      <c r="O27" s="3">
+        <v>12.198383538382499</v>
+      </c>
+      <c r="P27" s="3">
+        <v>80.409241098377606</v>
+      </c>
+      <c r="Q27" s="3">
+        <v>78.617068002496097</v>
+      </c>
+      <c r="R27" s="3">
+        <v>70.633412127131606</v>
+      </c>
+      <c r="S27" s="3">
+        <v>88.744262760997799</v>
+      </c>
+      <c r="T27" s="3">
+        <v>87.810996500577701</v>
+      </c>
+      <c r="U27" s="3">
+        <v>82.982947612957801</v>
+      </c>
+      <c r="V27" s="3">
+        <v>93.020765358798101</v>
+      </c>
+      <c r="W27" s="3">
+        <v>92.085499293044904</v>
+      </c>
+      <c r="X27" s="3">
+        <v>83.921160998291398</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A28" s="3">
+        <v>47.973012218272501</v>
+      </c>
+      <c r="B28" s="3">
+        <v>44.863680924374101</v>
+      </c>
+      <c r="C28" s="3">
+        <v>26.4017925008615</v>
+      </c>
+      <c r="D28" s="3">
+        <v>59.195837981364697</v>
+      </c>
+      <c r="E28" s="3">
+        <v>57.843186002404401</v>
+      </c>
+      <c r="F28" s="3">
+        <v>43.078718480735603</v>
+      </c>
+      <c r="G28" s="3">
+        <v>69.143411023483296</v>
+      </c>
+      <c r="H28" s="3">
+        <v>59.582896418028803</v>
+      </c>
+      <c r="I28" s="3">
+        <v>52.306163810195201</v>
+      </c>
+      <c r="J28" s="3">
+        <v>98.167515772427805</v>
+      </c>
+      <c r="K28" s="3">
+        <v>97.198694354783001</v>
+      </c>
+      <c r="L28" s="3">
+        <v>92.756968217815697</v>
+      </c>
+      <c r="M28" s="3">
+        <v>27.302904734642599</v>
+      </c>
+      <c r="N28" s="3">
+        <v>22.348070494021499</v>
+      </c>
+      <c r="O28" s="3">
+        <v>15.953032770797201</v>
+      </c>
+      <c r="P28" s="3">
+        <v>91.005281790043796</v>
+      </c>
+      <c r="Q28" s="3">
+        <v>85.179185576749802</v>
+      </c>
+      <c r="R28" s="3">
+        <v>62.783985942895903</v>
+      </c>
+      <c r="S28" s="3">
+        <v>96.138243304575894</v>
+      </c>
+      <c r="T28" s="3">
+        <v>92.7460984382124</v>
+      </c>
+      <c r="U28" s="3">
+        <v>80.804768883798801</v>
+      </c>
+      <c r="V28" s="3">
+        <v>92.211375771145697</v>
+      </c>
+      <c r="W28" s="3">
+        <v>87.666868199839698</v>
+      </c>
+      <c r="X28" s="3">
+        <v>64.964844935273803</v>
+      </c>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A29" s="3">
+        <v>52.515054308301004</v>
+      </c>
+      <c r="B29" s="3">
+        <v>42.0828535120922</v>
+      </c>
+      <c r="C29" s="3">
+        <v>8.8689792653009505</v>
+      </c>
+      <c r="D29" s="3">
+        <v>35.417686252823401</v>
+      </c>
+      <c r="E29" s="3">
+        <v>29.979612488504799</v>
+      </c>
+      <c r="F29" s="3">
+        <v>7.5999339759199103</v>
+      </c>
+      <c r="G29" s="3">
+        <v>87.811254050869096</v>
+      </c>
+      <c r="H29" s="3">
+        <v>58.689482470784597</v>
+      </c>
+      <c r="I29" s="3">
+        <v>36.138662476676799</v>
+      </c>
+      <c r="J29" s="3">
+        <v>96.517550476968907</v>
+      </c>
+      <c r="K29" s="3">
+        <v>88.623736087932102</v>
+      </c>
+      <c r="L29" s="3">
+        <v>57.047548346538299</v>
+      </c>
+      <c r="M29" s="3">
+        <v>63.991655783606802</v>
+      </c>
+      <c r="N29" s="3">
+        <v>35.973590384392701</v>
+      </c>
+      <c r="O29" s="3">
+        <v>11.162790916326101</v>
+      </c>
+      <c r="P29" s="3">
+        <v>83.984689762516993</v>
+      </c>
+      <c r="Q29" s="3">
+        <v>59.4310410495372</v>
+      </c>
+      <c r="R29" s="3">
+        <v>17.285038777169099</v>
+      </c>
+      <c r="S29" s="3">
+        <v>95.732270290409105</v>
+      </c>
+      <c r="T29" s="3">
+        <v>81.274549909917198</v>
+      </c>
+      <c r="U29" s="3">
+        <v>33.6770206015211</v>
+      </c>
+      <c r="V29" s="3">
+        <v>96.111102117334298</v>
+      </c>
+      <c r="W29" s="3">
+        <v>86.180317284069403</v>
+      </c>
+      <c r="X29" s="3">
+        <v>23.966140498706402</v>
+      </c>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A30" s="3">
+        <v>41.476911815801699</v>
+      </c>
+      <c r="B30" s="3">
+        <v>33.796849568140502</v>
+      </c>
+      <c r="C30" s="3">
+        <v>13.2862499869853</v>
+      </c>
+      <c r="D30" s="3">
+        <v>46.935037573559903</v>
+      </c>
+      <c r="E30" s="3">
+        <v>42.686093848838397</v>
+      </c>
+      <c r="F30" s="3">
+        <v>15.8981318999822</v>
+      </c>
+      <c r="G30" s="3">
+        <v>65.838607594936704</v>
+      </c>
+      <c r="H30" s="3">
+        <v>44.029617007465099</v>
+      </c>
+      <c r="I30" s="3">
+        <v>31.957319052255801</v>
+      </c>
+      <c r="J30" s="3">
+        <v>96.198236726946703</v>
+      </c>
+      <c r="K30" s="3">
+        <v>91.288099767842695</v>
+      </c>
+      <c r="L30" s="3">
+        <v>67.045917937138199</v>
+      </c>
+      <c r="M30" s="3">
+        <v>42.396150606742701</v>
+      </c>
+      <c r="N30" s="3">
+        <v>26.028544146603501</v>
+      </c>
+      <c r="O30" s="3">
+        <v>14.1339315929504</v>
+      </c>
+      <c r="P30" s="3">
+        <v>85.726225590671405</v>
+      </c>
+      <c r="Q30" s="3">
+        <v>67.822638585165095</v>
+      </c>
+      <c r="R30" s="3">
+        <v>30.8527822023254</v>
+      </c>
+      <c r="S30" s="3">
+        <v>92.912645470444005</v>
+      </c>
+      <c r="T30" s="3">
+        <v>81.431252036881304</v>
+      </c>
+      <c r="U30" s="3">
+        <v>45.484348115467199</v>
+      </c>
+      <c r="V30" s="3">
+        <v>90.094787775762796</v>
+      </c>
+      <c r="W30" s="3">
+        <v>78.335302524987995</v>
+      </c>
+      <c r="X30" s="3">
+        <v>33.681358067370297</v>
+      </c>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A31" s="3">
+        <v>24.895570601435502</v>
+      </c>
+      <c r="B31" s="3">
+        <v>19.338882548017001</v>
+      </c>
+      <c r="C31" s="3">
+        <v>7.6943876408749601</v>
+      </c>
+      <c r="D31" s="3">
+        <v>25.028144000077098</v>
+      </c>
+      <c r="E31" s="3">
+        <v>23.762984863989701</v>
+      </c>
+      <c r="F31" s="3">
+        <v>15.6996906822823</v>
+      </c>
+      <c r="G31" s="3">
+        <v>58.640648011781998</v>
+      </c>
+      <c r="H31" s="3">
+        <v>38.748159057437398</v>
+      </c>
+      <c r="I31" s="3">
+        <v>28.466863033873299</v>
+      </c>
+      <c r="J31" s="3">
+        <v>90.379956270449895</v>
+      </c>
+      <c r="K31" s="3">
+        <v>83.247903001777104</v>
+      </c>
+      <c r="L31" s="3">
+        <v>64.533624790046503</v>
+      </c>
+      <c r="M31" s="3">
+        <v>44.459737003222898</v>
+      </c>
+      <c r="N31" s="3">
+        <v>24.5587073559991</v>
+      </c>
+      <c r="O31" s="3">
+        <v>10.473106049293699</v>
+      </c>
+      <c r="P31" s="3">
+        <v>84.898884078555895</v>
+      </c>
+      <c r="Q31" s="3">
+        <v>65.019217540382897</v>
+      </c>
+      <c r="R31" s="3">
+        <v>30.549443115556802</v>
+      </c>
+      <c r="S31" s="3">
+        <v>88.882205217452494</v>
+      </c>
+      <c r="T31" s="3">
+        <v>75.002681259552503</v>
+      </c>
+      <c r="U31" s="3">
+        <v>41.188154516069297</v>
+      </c>
+      <c r="V31" s="3">
+        <v>86.283882607540605</v>
+      </c>
+      <c r="W31" s="3">
+        <v>70.643145365974206</v>
+      </c>
+      <c r="X31" s="3">
+        <v>30.7911414132913</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A32" s="3">
+        <v>79.387088434965094</v>
+      </c>
+      <c r="B32" s="3">
+        <v>66.693990740509705</v>
+      </c>
+      <c r="C32" s="3">
+        <v>12.395478367136</v>
+      </c>
+      <c r="D32" s="3">
+        <v>45.937063758783601</v>
+      </c>
+      <c r="E32" s="3">
+        <v>40.9378863011448</v>
+      </c>
+      <c r="F32" s="3">
+        <v>16.6632981599289</v>
+      </c>
+      <c r="G32" s="3">
+        <v>74.639209225700199</v>
+      </c>
+      <c r="H32" s="3">
+        <v>41.283360790774303</v>
+      </c>
+      <c r="I32" s="3">
+        <v>22.752883031301501</v>
+      </c>
+      <c r="J32" s="3">
+        <v>99.204813045847601</v>
+      </c>
+      <c r="K32" s="3">
+        <v>97.044299781425295</v>
+      </c>
+      <c r="L32" s="3">
+        <v>69.064134802913998</v>
+      </c>
+      <c r="M32" s="3">
+        <v>97.102770792676907</v>
+      </c>
+      <c r="N32" s="3">
+        <v>74.2372212167475</v>
+      </c>
+      <c r="O32" s="3">
+        <v>18.272849052506601</v>
+      </c>
+      <c r="P32" s="3">
+        <v>96.983478649143706</v>
+      </c>
+      <c r="Q32" s="3">
+        <v>78.025428309343695</v>
+      </c>
+      <c r="R32" s="3">
+        <v>18.032196658570001</v>
+      </c>
+      <c r="S32" s="3">
+        <v>98.372776197974204</v>
+      </c>
+      <c r="T32" s="3">
+        <v>88.657093839335502</v>
+      </c>
+      <c r="U32" s="3">
+        <v>29.247444244506401</v>
+      </c>
+      <c r="V32" s="3">
+        <v>98.307254746680798</v>
+      </c>
+      <c r="W32" s="3">
+        <v>87.069916100669303</v>
+      </c>
+      <c r="X32" s="3">
+        <v>18.089915631157002</v>
+      </c>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A33" s="3">
+        <v>65.114671344893907</v>
+      </c>
+      <c r="B33" s="3">
+        <v>60.002402108303002</v>
+      </c>
+      <c r="C33" s="3">
+        <v>21.348493803178599</v>
+      </c>
+      <c r="D33" s="3">
+        <v>29.357020543876899</v>
+      </c>
+      <c r="E33" s="3">
+        <v>27.5441579672773</v>
+      </c>
+      <c r="F33" s="3">
+        <v>13.982818045016399</v>
+      </c>
+      <c r="G33" s="3">
+        <v>80.296059782608694</v>
+      </c>
+      <c r="H33" s="3">
+        <v>61.8501358695652</v>
+      </c>
+      <c r="I33" s="3">
+        <v>47.064538043478301</v>
+      </c>
+      <c r="J33" s="3">
+        <v>97.295648375869703</v>
+      </c>
+      <c r="K33" s="3">
+        <v>94.808148632777801</v>
+      </c>
+      <c r="L33" s="3">
+        <v>83.233985769365603</v>
+      </c>
+      <c r="M33" s="3">
+        <v>84.308420878718906</v>
+      </c>
+      <c r="N33" s="3">
+        <v>73.617574461929806</v>
+      </c>
+      <c r="O33" s="3">
+        <v>38.395611797252698</v>
+      </c>
+      <c r="P33" s="3">
+        <v>95.477951366618498</v>
+      </c>
+      <c r="Q33" s="3">
+        <v>87.467954943978995</v>
+      </c>
+      <c r="R33" s="3">
+        <v>45.482829741873502</v>
+      </c>
+      <c r="S33" s="3">
+        <v>96.696080822846994</v>
+      </c>
+      <c r="T33" s="3">
+        <v>90.905998145273799</v>
+      </c>
+      <c r="U33" s="3">
+        <v>67.112150134080395</v>
+      </c>
+      <c r="V33" s="3">
+        <v>97.234065728353002</v>
+      </c>
+      <c r="W33" s="3">
+        <v>92.901796445761505</v>
+      </c>
+      <c r="X33" s="3">
+        <v>53.278837886386199</v>
+      </c>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A34" s="3">
+        <v>44.922591014458597</v>
+      </c>
+      <c r="B34" s="3">
+        <v>38.666254654266403</v>
+      </c>
+      <c r="C34" s="3">
+        <v>12.3711663715925</v>
+      </c>
+      <c r="D34" s="3">
+        <v>35.032789770848503</v>
+      </c>
+      <c r="E34" s="3">
+        <v>31.628650236781699</v>
+      </c>
+      <c r="F34" s="3">
+        <v>13.039663417152701</v>
+      </c>
+      <c r="G34" s="3">
+        <v>78.972873082287293</v>
+      </c>
+      <c r="H34" s="3">
+        <v>57.723152022315197</v>
+      </c>
+      <c r="I34" s="3">
+        <v>41.441422594142303</v>
+      </c>
+      <c r="J34" s="3">
+        <v>96.195606885758096</v>
+      </c>
+      <c r="K34" s="3">
+        <v>90.448202567649702</v>
+      </c>
+      <c r="L34" s="3">
+        <v>70.448137808561995</v>
+      </c>
+      <c r="M34" s="3">
+        <v>73.2174376520165</v>
+      </c>
+      <c r="N34" s="3">
+        <v>55.4711477970475</v>
+      </c>
+      <c r="O34" s="3">
+        <v>22.422499500679098</v>
+      </c>
+      <c r="P34" s="3">
+        <v>92.767197996085798</v>
+      </c>
+      <c r="Q34" s="3">
+        <v>80.833614188348804</v>
+      </c>
+      <c r="R34" s="3">
+        <v>35.285351598892802</v>
+      </c>
+      <c r="S34" s="3">
+        <v>94.154359581393607</v>
+      </c>
+      <c r="T34" s="3">
+        <v>86.042605451026105</v>
+      </c>
+      <c r="U34" s="3">
+        <v>56.468686815009697</v>
+      </c>
+      <c r="V34" s="3">
+        <v>94.241472495584901</v>
+      </c>
+      <c r="W34" s="3">
+        <v>86.721466289092007</v>
+      </c>
+      <c r="X34" s="3">
+        <v>41.109651019121799</v>
+      </c>
+    </row>
+    <row r="35" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A35" s="3">
+        <v>50.368073926776297</v>
+      </c>
+      <c r="B35" s="3">
+        <v>48.129516606979898</v>
+      </c>
+      <c r="C35" s="3">
+        <v>36.132422711253902</v>
+      </c>
+      <c r="D35" s="3">
+        <v>13.0024407609643</v>
+      </c>
+      <c r="E35" s="3">
+        <v>12.2286015031997</v>
+      </c>
+      <c r="F35" s="3">
+        <v>10.321669528146501</v>
+      </c>
+      <c r="G35" s="3">
+        <v>83.507504690431503</v>
+      </c>
+      <c r="H35" s="3">
+        <v>77.521575984990605</v>
+      </c>
+      <c r="I35" s="3">
+        <v>71.7823639774859</v>
+      </c>
+      <c r="J35" s="3">
+        <v>94.519655734180205</v>
+      </c>
+      <c r="K35" s="3">
+        <v>92.199583198579504</v>
+      </c>
+      <c r="L35" s="3">
+        <v>84.516829323441897</v>
+      </c>
+      <c r="M35" s="3">
+        <v>72.237996095930995</v>
+      </c>
+      <c r="N35" s="3">
+        <v>65.263626982126297</v>
+      </c>
+      <c r="O35" s="3">
+        <v>55.116611653968803</v>
+      </c>
+      <c r="P35" s="3">
+        <v>91.903574224848896</v>
+      </c>
+      <c r="Q35" s="3">
+        <v>86.636942052635902</v>
+      </c>
+      <c r="R35" s="3">
+        <v>72.739875210991499</v>
+      </c>
+      <c r="S35" s="3">
+        <v>96.361068527274995</v>
+      </c>
+      <c r="T35" s="3">
+        <v>94.078454017960595</v>
+      </c>
+      <c r="U35" s="3">
+        <v>84.567626234581894</v>
+      </c>
+      <c r="V35" s="3">
+        <v>97.584460377514304</v>
+      </c>
+      <c r="W35" s="3">
+        <v>95.281680019464702</v>
+      </c>
+      <c r="X35" s="3">
+        <v>81.033943970601399</v>
+      </c>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A36" s="3">
+        <v>61.515128103959</v>
+      </c>
+      <c r="B36" s="3">
+        <v>56.183815022975097</v>
+      </c>
+      <c r="C36" s="3">
+        <v>24.237389065069198</v>
+      </c>
+      <c r="D36" s="3">
+        <v>26.021565567336701</v>
+      </c>
+      <c r="E36" s="3">
+        <v>24.266825845411301</v>
+      </c>
+      <c r="F36" s="3">
+        <v>10.567192726688599</v>
+      </c>
+      <c r="G36" s="3">
+        <v>83.324596774193594</v>
+      </c>
+      <c r="H36" s="3">
+        <v>64.881048387096797</v>
+      </c>
+      <c r="I36" s="3">
+        <v>50.058467741935502</v>
+      </c>
+      <c r="J36" s="3">
+        <v>98.644828826423705</v>
+      </c>
+      <c r="K36" s="3">
+        <v>96.606549859097498</v>
+      </c>
+      <c r="L36" s="3">
+        <v>85.186706775925003</v>
+      </c>
+      <c r="M36" s="3">
+        <v>71.055073401554395</v>
+      </c>
+      <c r="N36" s="3">
+        <v>57.0576907839312</v>
+      </c>
+      <c r="O36" s="3">
+        <v>33.125659977977399</v>
+      </c>
+      <c r="P36" s="3">
+        <v>86.718201868680396</v>
+      </c>
+      <c r="Q36" s="3">
+        <v>75.524247659832497</v>
+      </c>
+      <c r="R36" s="3">
+        <v>39.889922808720598</v>
+      </c>
+      <c r="S36" s="3">
+        <v>96.149169020274996</v>
+      </c>
+      <c r="T36" s="3">
+        <v>90.5684750142361</v>
+      </c>
+      <c r="U36" s="3">
+        <v>62.276653035329701</v>
+      </c>
+      <c r="V36" s="3">
+        <v>95.761265459593702</v>
+      </c>
+      <c r="W36" s="3">
+        <v>89.880744566530396</v>
+      </c>
+      <c r="X36" s="3">
+        <v>51.4272521632994</v>
+      </c>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A37" s="3">
+        <v>66.446882062849099</v>
+      </c>
+      <c r="B37" s="3">
+        <v>58.4224300527625</v>
+      </c>
+      <c r="C37" s="3">
+        <v>23.7214804255558</v>
+      </c>
+      <c r="D37" s="3">
+        <v>43.996118250678798</v>
+      </c>
+      <c r="E37" s="3">
+        <v>39.099519129580798</v>
+      </c>
+      <c r="F37" s="3">
+        <v>17.272160722326898</v>
+      </c>
+      <c r="G37" s="3">
+        <v>89.521932424422005</v>
+      </c>
+      <c r="H37" s="3">
+        <v>64.915678719620601</v>
+      </c>
+      <c r="I37" s="3">
+        <v>46.8055720213397</v>
+      </c>
+      <c r="J37" s="3">
+        <v>97.149214747166994</v>
+      </c>
+      <c r="K37" s="3">
+        <v>91.685295062182703</v>
+      </c>
+      <c r="L37" s="3">
+        <v>65.274518356648997</v>
+      </c>
+      <c r="M37" s="3">
+        <v>69.830550559817198</v>
+      </c>
+      <c r="N37" s="3">
+        <v>47.215557789847402</v>
+      </c>
+      <c r="O37" s="3">
+        <v>26.128872927512099</v>
+      </c>
+      <c r="P37" s="3">
+        <v>86.0427005372797</v>
+      </c>
+      <c r="Q37" s="3">
+        <v>65.746548421265899</v>
+      </c>
+      <c r="R37" s="3">
+        <v>34.696435061272098</v>
+      </c>
+      <c r="S37" s="3">
+        <v>96.421534405657397</v>
+      </c>
+      <c r="T37" s="3">
+        <v>86.096751522508001</v>
+      </c>
+      <c r="U37" s="3">
+        <v>49.662565313542103</v>
+      </c>
+      <c r="V37" s="3">
+        <v>96.419099088410604</v>
+      </c>
+      <c r="W37" s="3">
+        <v>88.432623050040903</v>
+      </c>
+      <c r="X37" s="3">
+        <v>42.219058045312799</v>
+      </c>
+    </row>
+    <row r="38" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A38" s="3">
+        <v>53.105433072572303</v>
+      </c>
+      <c r="B38" s="3">
+        <v>46.172041015397603</v>
+      </c>
+      <c r="C38" s="3">
+        <v>2.8074250585810199</v>
+      </c>
+      <c r="D38" s="3">
+        <v>6.72660645988657</v>
+      </c>
+      <c r="E38" s="3">
+        <v>4.4049295999886597</v>
+      </c>
+      <c r="F38" s="3">
+        <v>1.3138473381971301</v>
+      </c>
+      <c r="G38" s="3">
+        <v>80.044506258692607</v>
+      </c>
+      <c r="H38" s="3">
+        <v>54.815020862308799</v>
+      </c>
+      <c r="I38" s="3">
+        <v>34.417246175243399</v>
+      </c>
+      <c r="J38" s="3">
+        <v>92.765062264851593</v>
+      </c>
+      <c r="K38" s="3">
+        <v>83.831674643021202</v>
+      </c>
+      <c r="L38" s="3">
+        <v>67.856585033624398</v>
+      </c>
+      <c r="M38" s="3">
+        <v>24.697797983807298</v>
+      </c>
+      <c r="N38" s="3">
+        <v>10.052397260456599</v>
+      </c>
+      <c r="O38" s="3">
+        <v>1.11660670462676</v>
+      </c>
+      <c r="P38" s="3">
+        <v>89.426122090613603</v>
+      </c>
+      <c r="Q38" s="3">
+        <v>74.520136787107106</v>
+      </c>
+      <c r="R38" s="3">
+        <v>11.4955801634192</v>
+      </c>
+      <c r="S38" s="3">
+        <v>94.168819292707695</v>
+      </c>
+      <c r="T38" s="3">
+        <v>83.552155852328895</v>
+      </c>
+      <c r="U38" s="3">
+        <v>43.1407650667147</v>
+      </c>
+      <c r="V38" s="3">
+        <v>90.156524284806906</v>
+      </c>
+      <c r="W38" s="3">
+        <v>76.288449684739007</v>
+      </c>
+      <c r="X38" s="3">
+        <v>12.5098397823126</v>
+      </c>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A39" s="3">
+        <v>59.217514992679902</v>
+      </c>
+      <c r="B39" s="3">
+        <v>52.801947492350102</v>
+      </c>
+      <c r="C39" s="3">
+        <v>16.3367066016338</v>
+      </c>
+      <c r="D39" s="3">
+        <v>62.804496541770099</v>
+      </c>
+      <c r="E39" s="3">
+        <v>59.588118052083303</v>
+      </c>
+      <c r="F39" s="3">
+        <v>28.8068831335593</v>
+      </c>
+      <c r="G39" s="3">
+        <v>73.583481843441604</v>
+      </c>
+      <c r="H39" s="3">
+        <v>52.9097058541726</v>
+      </c>
+      <c r="I39" s="3">
+        <v>37.646239340806702</v>
+      </c>
+      <c r="J39" s="3">
+        <v>99.226257417116599</v>
+      </c>
+      <c r="K39" s="3">
+        <v>97.068451452819204</v>
+      </c>
+      <c r="L39" s="3">
+        <v>83.369617610025102</v>
+      </c>
+      <c r="M39" s="3">
+        <v>35.320925638865297</v>
+      </c>
+      <c r="N39" s="3">
+        <v>23.819046773359499</v>
+      </c>
+      <c r="O39" s="3">
+        <v>8.4767004776977402</v>
+      </c>
+      <c r="P39" s="3">
+        <v>86.954468054954901</v>
+      </c>
+      <c r="Q39" s="3">
+        <v>70.821235640550796</v>
+      </c>
+      <c r="R39" s="3">
+        <v>32.870402243446897</v>
+      </c>
+      <c r="S39" s="3">
+        <v>95.548202351000398</v>
+      </c>
+      <c r="T39" s="3">
+        <v>86.995694850260094</v>
+      </c>
+      <c r="U39" s="3">
+        <v>56.094377704651997</v>
+      </c>
+      <c r="V39" s="3">
+        <v>87.684156963806103</v>
+      </c>
+      <c r="W39" s="3">
+        <v>77.3164211818453</v>
+      </c>
+      <c r="X39" s="3">
+        <v>33.9141869192729</v>
+      </c>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A40" s="3">
+        <v>49.464948603291099</v>
+      </c>
+      <c r="B40" s="3">
+        <v>43.091856063416301</v>
+      </c>
+      <c r="C40" s="3">
+        <v>14.1619357290731</v>
+      </c>
+      <c r="D40" s="3">
+        <v>53.500950575787499</v>
+      </c>
+      <c r="E40" s="3">
+        <v>50.170992075621903</v>
+      </c>
+      <c r="F40" s="3">
+        <v>23.9036995649174</v>
+      </c>
+      <c r="G40" s="3">
+        <v>69.839769813462794</v>
+      </c>
+      <c r="H40" s="3">
+        <v>50.4460059895477</v>
+      </c>
+      <c r="I40" s="3">
+        <v>36.697332106715699</v>
+      </c>
+      <c r="J40" s="3">
+        <v>98.433939069847497</v>
+      </c>
+      <c r="K40" s="3">
+        <v>95.523632715626604</v>
+      </c>
+      <c r="L40" s="3">
+        <v>80.369468855558296</v>
+      </c>
+      <c r="M40" s="3">
+        <v>34.704767117387597</v>
+      </c>
+      <c r="N40" s="3">
+        <v>22.252713801987699</v>
+      </c>
+      <c r="O40" s="3">
+        <v>7.90091712974011</v>
+      </c>
+      <c r="P40" s="3">
+        <v>84.926220239159306</v>
+      </c>
+      <c r="Q40" s="3">
+        <v>69.002556974589993</v>
+      </c>
+      <c r="R40" s="3">
+        <v>35.187110375082902</v>
+      </c>
+      <c r="S40" s="3">
+        <v>94.378607471764695</v>
+      </c>
+      <c r="T40" s="3">
+        <v>85.135783718689297</v>
+      </c>
+      <c r="U40" s="3">
+        <v>54.782614673947897</v>
+      </c>
+      <c r="V40" s="3">
+        <v>85.238586126630906</v>
+      </c>
+      <c r="W40" s="3">
+        <v>74.924706068307898</v>
+      </c>
+      <c r="X40" s="3">
+        <v>34.107361118275797</v>
+      </c>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A41" s="3">
+        <v>44.7229735569978</v>
+      </c>
+      <c r="B41" s="3">
+        <v>38.915889133127003</v>
+      </c>
+      <c r="C41" s="3">
+        <v>14.5094376966161</v>
+      </c>
+      <c r="D41" s="3">
+        <v>44.7027703902437</v>
+      </c>
+      <c r="E41" s="3">
+        <v>41.713644359212601</v>
+      </c>
+      <c r="F41" s="3">
+        <v>20.461676342531302</v>
+      </c>
+      <c r="G41" s="3">
+        <v>69.572640914390604</v>
+      </c>
+      <c r="H41" s="3">
+        <v>51.095070624438499</v>
+      </c>
+      <c r="I41" s="3">
+        <v>38.088801391463903</v>
+      </c>
+      <c r="J41" s="3">
+        <v>97.700644913638797</v>
+      </c>
+      <c r="K41" s="3">
+        <v>94.040639266629697</v>
+      </c>
+      <c r="L41" s="3">
+        <v>78.380633403538894</v>
+      </c>
+      <c r="M41" s="3">
+        <v>37.374423080361801</v>
+      </c>
+      <c r="N41" s="3">
+        <v>24.569656772402102</v>
+      </c>
+      <c r="O41" s="3">
+        <v>9.7532356867727792</v>
+      </c>
+      <c r="P41" s="3">
+        <v>85.086411724990796</v>
+      </c>
+      <c r="Q41" s="3">
+        <v>70.410917112436294</v>
+      </c>
+      <c r="R41" s="3">
+        <v>38.815456856586103</v>
+      </c>
+      <c r="S41" s="3">
+        <v>93.505284760439295</v>
+      </c>
+      <c r="T41" s="3">
+        <v>84.505973333956206</v>
+      </c>
+      <c r="U41" s="3">
+        <v>56.045898995114399</v>
+      </c>
+      <c r="V41" s="3">
+        <v>85.265112675765295</v>
+      </c>
+      <c r="W41" s="3">
+        <v>76.221405374244</v>
+      </c>
+      <c r="X41" s="3">
+        <v>37.449740708607798</v>
+      </c>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A42" s="3">
+        <v>39.093923732180002</v>
+      </c>
+      <c r="B42" s="3">
+        <v>33.9929537300834</v>
+      </c>
+      <c r="C42" s="3">
+        <v>15.3811004443802</v>
+      </c>
+      <c r="D42" s="3">
+        <v>35.877051072802701</v>
+      </c>
+      <c r="E42" s="3">
+        <v>33.322963177297297</v>
+      </c>
+      <c r="F42" s="3">
+        <v>18.284999903876098</v>
+      </c>
+      <c r="G42" s="3">
+        <v>68.211532280933895</v>
+      </c>
+      <c r="H42" s="3">
+        <v>51.852651479345901</v>
+      </c>
+      <c r="I42" s="3">
+        <v>40.608242745060998</v>
+      </c>
+      <c r="J42" s="3">
+        <v>97.001844389341898</v>
+      </c>
+      <c r="K42" s="3">
+        <v>93.039726075598296</v>
+      </c>
+      <c r="L42" s="3">
+        <v>78.495983403470703</v>
+      </c>
+      <c r="M42" s="3">
+        <v>37.551200294222703</v>
+      </c>
+      <c r="N42" s="3">
+        <v>26.214121546912999</v>
+      </c>
+      <c r="O42" s="3">
+        <v>12.567338589466701</v>
+      </c>
+      <c r="P42" s="3">
+        <v>85.058582602833397</v>
+      </c>
+      <c r="Q42" s="3">
+        <v>72.131079369484695</v>
+      </c>
+      <c r="R42" s="3">
+        <v>44.226693039248602</v>
+      </c>
+      <c r="S42" s="3">
+        <v>92.371291274467694</v>
+      </c>
+      <c r="T42" s="3">
+        <v>83.819386943437394</v>
+      </c>
+      <c r="U42" s="3">
+        <v>58.173577810951301</v>
+      </c>
+      <c r="V42" s="3">
+        <v>84.831367707022494</v>
+      </c>
+      <c r="W42" s="3">
+        <v>76.824759384896893</v>
+      </c>
+      <c r="X42" s="3">
+        <v>42.822175158580997</v>
+      </c>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A43" s="3">
+        <v>33.481690118397204</v>
+      </c>
+      <c r="B43" s="3">
+        <v>31.154694129098601</v>
+      </c>
+      <c r="C43" s="3">
+        <v>23.176450863523399</v>
+      </c>
+      <c r="D43" s="3">
+        <v>29.713575869215401</v>
+      </c>
+      <c r="E43" s="3">
+        <v>28.617379699203202</v>
+      </c>
+      <c r="F43" s="3">
+        <v>22.7243473217979</v>
+      </c>
+      <c r="G43" s="3">
+        <v>63.791097843860499</v>
+      </c>
+      <c r="H43" s="3">
+        <v>53.824732859261502</v>
+      </c>
+      <c r="I43" s="3">
+        <v>47.357835494543103</v>
+      </c>
+      <c r="J43" s="3">
+        <v>94.311637289934794</v>
+      </c>
+      <c r="K43" s="3">
+        <v>91.0489466647239</v>
+      </c>
+      <c r="L43" s="3">
+        <v>81.935856705838304</v>
+      </c>
+      <c r="M43" s="3">
+        <v>35.522820142897501</v>
+      </c>
+      <c r="N43" s="3">
+        <v>28.7617891635477</v>
+      </c>
+      <c r="O43" s="3">
+        <v>21.965886762190699</v>
+      </c>
+      <c r="P43" s="3">
+        <v>84.609969476586798</v>
+      </c>
+      <c r="Q43" s="3">
+        <v>76.958349040608795</v>
+      </c>
+      <c r="R43" s="3">
+        <v>61.402851112614698</v>
+      </c>
+      <c r="S43" s="3">
+        <v>88.292365925678794</v>
+      </c>
+      <c r="T43" s="3">
+        <v>82.214685243189606</v>
+      </c>
+      <c r="U43" s="3">
+        <v>68.150764492325493</v>
+      </c>
+      <c r="V43" s="3">
+        <v>82.998957992339001</v>
+      </c>
+      <c r="W43" s="3">
+        <v>77.940082643151698</v>
+      </c>
+      <c r="X43" s="3">
+        <v>59.201737846980201</v>
+      </c>
+    </row>
+    <row r="44" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A44" s="3">
+        <v>47.098018188697601</v>
+      </c>
+      <c r="B44" s="3">
+        <v>40.8443146518715</v>
+      </c>
+      <c r="C44" s="3">
+        <v>12.9648084333756</v>
+      </c>
+      <c r="D44" s="3">
+        <v>50.503002122069098</v>
+      </c>
+      <c r="E44" s="3">
+        <v>47.345681201139101</v>
+      </c>
+      <c r="F44" s="3">
+        <v>22.648968666837298</v>
+      </c>
+      <c r="G44" s="3">
+        <v>69.3039418416801</v>
+      </c>
+      <c r="H44" s="3">
+        <v>48.735379644588001</v>
+      </c>
+      <c r="I44" s="3">
+        <v>34.427483037156698</v>
+      </c>
+      <c r="J44" s="3">
+        <v>97.981818172716601</v>
+      </c>
+      <c r="K44" s="3">
+        <v>94.449756836709597</v>
+      </c>
+      <c r="L44" s="3">
+        <v>78.358884490613704</v>
+      </c>
+      <c r="M44" s="3">
+        <v>35.402096524006197</v>
+      </c>
+      <c r="N44" s="3">
+        <v>22.6402252958795</v>
+      </c>
+      <c r="O44" s="3">
+        <v>8.1409326765486192</v>
+      </c>
+      <c r="P44" s="3">
+        <v>83.685239728834702</v>
+      </c>
+      <c r="Q44" s="3">
+        <v>67.235321952887602</v>
+      </c>
+      <c r="R44" s="3">
+        <v>33.144201151157098</v>
+      </c>
+      <c r="S44" s="3">
+        <v>93.054638178440896</v>
+      </c>
+      <c r="T44" s="3">
+        <v>83.003877273768296</v>
+      </c>
+      <c r="U44" s="3">
+        <v>51.922562428830197</v>
+      </c>
+      <c r="V44" s="3">
+        <v>84.143947588173006</v>
+      </c>
+      <c r="W44" s="3">
+        <v>73.575961139641905</v>
+      </c>
+      <c r="X44" s="3">
+        <v>32.161468932980497</v>
+      </c>
+    </row>
+    <row r="45" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A45" s="3">
+        <v>43.179013973835502</v>
+      </c>
+      <c r="B45" s="3">
+        <v>39.971792454873203</v>
+      </c>
+      <c r="C45" s="3">
+        <v>24.486713074181299</v>
+      </c>
+      <c r="D45" s="3">
+        <v>36.835495870869501</v>
+      </c>
+      <c r="E45" s="3">
+        <v>35.181605699871596</v>
+      </c>
+      <c r="F45" s="3">
+        <v>23.9265325853127</v>
+      </c>
+      <c r="G45" s="3">
+        <v>68.523699356731697</v>
+      </c>
+      <c r="H45" s="3">
+        <v>56.834969717488597</v>
+      </c>
+      <c r="I45" s="3">
+        <v>48.369493661362498</v>
+      </c>
+      <c r="J45" s="3">
+        <v>96.287076745620197</v>
+      </c>
+      <c r="K45" s="3">
+        <v>93.963286955339697</v>
+      </c>
+      <c r="L45" s="3">
+        <v>85.430810016330895</v>
+      </c>
+      <c r="M45" s="3">
+        <v>37.4980818256277</v>
+      </c>
+      <c r="N45" s="3">
+        <v>30.137422066287101</v>
+      </c>
+      <c r="O45" s="3">
+        <v>19.883365878156098</v>
+      </c>
+      <c r="P45" s="3">
+        <v>89.088914110757898</v>
+      </c>
+      <c r="Q45" s="3">
+        <v>81.524775390614195</v>
+      </c>
+      <c r="R45" s="3">
+        <v>60.827398131573098</v>
+      </c>
+      <c r="S45" s="3">
+        <v>92.835899476221101</v>
+      </c>
+      <c r="T45" s="3">
+        <v>88.245695852604598</v>
+      </c>
+      <c r="U45" s="3">
+        <v>72.508833142434298</v>
+      </c>
+      <c r="V45" s="3">
+        <v>87.863835550295406</v>
+      </c>
+      <c r="W45" s="3">
+        <v>83.286812931876796</v>
+      </c>
+      <c r="X45" s="3">
+        <v>60.041757252780897</v>
+      </c>
+    </row>
+    <row r="46" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A46" s="3">
+        <v>61.9790813912104</v>
+      </c>
+      <c r="B46" s="3">
+        <v>55.244628610563701</v>
+      </c>
+      <c r="C46" s="3">
+        <v>15.9295937890174</v>
+      </c>
+      <c r="D46" s="3">
+        <v>64.982324618476</v>
+      </c>
+      <c r="E46" s="3">
+        <v>61.619659768036499</v>
+      </c>
+      <c r="F46" s="3">
+        <v>29.331346170843599</v>
+      </c>
+      <c r="G46" s="3">
+        <v>74.508178093040897</v>
+      </c>
+      <c r="H46" s="3">
+        <v>52.601804345580398</v>
+      </c>
+      <c r="I46" s="3">
+        <v>36.423298095795602</v>
+      </c>
+      <c r="J46" s="3">
+        <v>99.419648251499893</v>
+      </c>
+      <c r="K46" s="3">
+        <v>97.332285145776495</v>
+      </c>
+      <c r="L46" s="3">
+        <v>83.609527784261999</v>
+      </c>
+      <c r="M46" s="3">
+        <v>35.861246656836499</v>
+      </c>
+      <c r="N46" s="3">
+        <v>24.100619208723899</v>
+      </c>
+      <c r="O46" s="3">
+        <v>7.9437195598066896</v>
+      </c>
+      <c r="P46" s="3">
+        <v>87.085034167996199</v>
+      </c>
+      <c r="Q46" s="3">
+        <v>70.362043366851296</v>
+      </c>
+      <c r="R46" s="3">
+        <v>30.685562238723801</v>
+      </c>
+      <c r="S46" s="3">
+        <v>95.776665967672002</v>
+      </c>
+      <c r="T46" s="3">
+        <v>87.148618072777893</v>
+      </c>
+      <c r="U46" s="3">
+        <v>55.079409797433598</v>
+      </c>
+      <c r="V46" s="3">
+        <v>87.994862849893806</v>
+      </c>
+      <c r="W46" s="3">
+        <v>77.276258760615505</v>
+      </c>
+      <c r="X46" s="3">
+        <v>32.227766046747803</v>
+      </c>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A47" s="3">
+        <v>51.201884065619197</v>
+      </c>
+      <c r="B47" s="3">
+        <v>44.623271204511802</v>
+      </c>
+      <c r="C47" s="3">
+        <v>12.9157008087651</v>
+      </c>
+      <c r="D47" s="3">
+        <v>58.016676735850503</v>
+      </c>
+      <c r="E47" s="3">
+        <v>54.682380794270799</v>
+      </c>
+      <c r="F47" s="3">
+        <v>25.154690089513</v>
+      </c>
+      <c r="G47" s="3">
+        <v>70.074609473419002</v>
+      </c>
+      <c r="H47" s="3">
+        <v>49.391880826404602</v>
+      </c>
+      <c r="I47" s="3">
+        <v>34.612433862433903</v>
+      </c>
+      <c r="J47" s="3">
+        <v>98.757702983131793</v>
+      </c>
+      <c r="K47" s="3">
+        <v>96.075163647536399</v>
+      </c>
+      <c r="L47" s="3">
+        <v>80.6602902609023</v>
+      </c>
+      <c r="M47" s="3">
+        <v>33.444713083497597</v>
+      </c>
+      <c r="N47" s="3">
+        <v>20.9814622056365</v>
+      </c>
+      <c r="O47" s="3">
+        <v>6.5810859872917504</v>
+      </c>
+      <c r="P47" s="3">
+        <v>84.614618462550695</v>
+      </c>
+      <c r="Q47" s="3">
+        <v>67.436079374054003</v>
+      </c>
+      <c r="R47" s="3">
+        <v>31.043904516240602</v>
+      </c>
+      <c r="S47" s="3">
+        <v>94.572670350347906</v>
+      </c>
+      <c r="T47" s="3">
+        <v>84.766180919128402</v>
+      </c>
+      <c r="U47" s="3">
+        <v>52.252155651821298</v>
+      </c>
+      <c r="V47" s="3">
+        <v>85.353424656889302</v>
+      </c>
+      <c r="W47" s="3">
+        <v>74.237308929192807</v>
+      </c>
+      <c r="X47" s="3">
+        <v>30.640352823690101</v>
+      </c>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A48" s="3">
+        <v>45.833605648748097</v>
+      </c>
+      <c r="B48" s="3">
+        <v>39.094393378310798</v>
+      </c>
+      <c r="C48" s="3">
+        <v>11.6710918209137</v>
+      </c>
+      <c r="D48" s="3">
+        <v>50.7394017828627</v>
+      </c>
+      <c r="E48" s="3">
+        <v>47.273402008568397</v>
+      </c>
+      <c r="F48" s="3">
+        <v>21.548502339823099</v>
+      </c>
+      <c r="G48" s="3">
+        <v>68.653063153914005</v>
+      </c>
+      <c r="H48" s="3">
+        <v>47.756870036556201</v>
+      </c>
+      <c r="I48" s="3">
+        <v>33.462687507878499</v>
+      </c>
+      <c r="J48" s="3">
+        <v>98.181784409523303</v>
+      </c>
+      <c r="K48" s="3">
+        <v>94.591175122134402</v>
+      </c>
+      <c r="L48" s="3">
+        <v>77.6130638893775</v>
+      </c>
+      <c r="M48" s="3">
+        <v>34.774396408509602</v>
+      </c>
+      <c r="N48" s="3">
+        <v>21.146634419683298</v>
+      </c>
+      <c r="O48" s="3">
+        <v>6.7988416055574099</v>
+      </c>
+      <c r="P48" s="3">
+        <v>82.964920272368104</v>
+      </c>
+      <c r="Q48" s="3">
+        <v>65.960696609533201</v>
+      </c>
+      <c r="R48" s="3">
+        <v>31.9319892996573</v>
+      </c>
+      <c r="S48" s="3">
+        <v>93.245754653718606</v>
+      </c>
+      <c r="T48" s="3">
+        <v>82.831637287221795</v>
+      </c>
+      <c r="U48" s="3">
+        <v>50.862129988055301</v>
+      </c>
+      <c r="V48" s="3">
+        <v>83.524510780059103</v>
+      </c>
+      <c r="W48" s="3">
+        <v>72.453516006402296</v>
+      </c>
+      <c r="X48" s="3">
+        <v>30.321201689915501</v>
+      </c>
+    </row>
+    <row r="49" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A49" s="3">
+        <v>41.487557947701603</v>
+      </c>
+      <c r="B49" s="3">
+        <v>35.1172718768197</v>
+      </c>
+      <c r="C49" s="3">
+        <v>10.962189864369501</v>
+      </c>
+      <c r="D49" s="3">
+        <v>43.529790152498897</v>
+      </c>
+      <c r="E49" s="3">
+        <v>40.2755960637855</v>
+      </c>
+      <c r="F49" s="3">
+        <v>18.544628258193899</v>
+      </c>
+      <c r="G49" s="3">
+        <v>68.249277433182897</v>
+      </c>
+      <c r="H49" s="3">
+        <v>47.488650017861197</v>
+      </c>
+      <c r="I49" s="3">
+        <v>33.195498977040202</v>
+      </c>
+      <c r="J49" s="3">
+        <v>97.530372680008398</v>
+      </c>
+      <c r="K49" s="3">
+        <v>93.299377945518202</v>
+      </c>
+      <c r="L49" s="3">
+        <v>75.468862416711104</v>
+      </c>
+      <c r="M49" s="3">
+        <v>36.663737339810297</v>
+      </c>
+      <c r="N49" s="3">
+        <v>22.683668646427002</v>
+      </c>
+      <c r="O49" s="3">
+        <v>7.4056821137641</v>
+      </c>
+      <c r="P49" s="3">
+        <v>83.1885935146245</v>
+      </c>
+      <c r="Q49" s="3">
+        <v>66.404015839562902</v>
+      </c>
+      <c r="R49" s="3">
+        <v>33.470065297067102</v>
+      </c>
+      <c r="S49" s="3">
+        <v>92.281749864229894</v>
+      </c>
+      <c r="T49" s="3">
+        <v>81.987219712724794</v>
+      </c>
+      <c r="U49" s="3">
+        <v>50.382793581421403</v>
+      </c>
+      <c r="V49" s="3">
+        <v>83.157490764716101</v>
+      </c>
+      <c r="W49" s="3">
+        <v>72.885916405896197</v>
+      </c>
+      <c r="X49" s="3">
+        <v>31.397287323923202</v>
+      </c>
+    </row>
+    <row r="50" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A50" s="3">
+        <v>34.014088196321197</v>
+      </c>
+      <c r="B50" s="3">
+        <v>29.231685479765002</v>
+      </c>
+      <c r="C50" s="3">
+        <v>13.2434616819192</v>
+      </c>
+      <c r="D50" s="3">
+        <v>33.969059746817301</v>
+      </c>
+      <c r="E50" s="3">
+        <v>31.6331726453048</v>
+      </c>
+      <c r="F50" s="3">
+        <v>18.182019831001501</v>
+      </c>
+      <c r="G50" s="3">
+        <v>65.407387375922596</v>
+      </c>
+      <c r="H50" s="3">
+        <v>46.709118096207703</v>
+      </c>
+      <c r="I50" s="3">
+        <v>34.577596080427597</v>
+      </c>
+      <c r="J50" s="3">
+        <v>95.886539172178701</v>
+      </c>
+      <c r="K50" s="3">
+        <v>90.687077447712497</v>
+      </c>
+      <c r="L50" s="3">
+        <v>74.039896434290299</v>
+      </c>
+      <c r="M50" s="3">
+        <v>36.427726083989697</v>
+      </c>
+      <c r="N50" s="3">
+        <v>24.404843169144701</v>
+      </c>
+      <c r="O50" s="3">
+        <v>12.1393046621136</v>
+      </c>
+      <c r="P50" s="3">
+        <v>80.382901654946195</v>
+      </c>
+      <c r="Q50" s="3">
+        <v>65.905160558700402</v>
+      </c>
+      <c r="R50" s="3">
+        <v>38.901866700519797</v>
+      </c>
+      <c r="S50" s="3">
+        <v>89.150843714897107</v>
+      </c>
+      <c r="T50" s="3">
+        <v>77.972749657136703</v>
+      </c>
+      <c r="U50" s="3">
+        <v>50.896750349778699</v>
+      </c>
+      <c r="V50" s="3">
+        <v>80.447857374899101</v>
+      </c>
+      <c r="W50" s="3">
+        <v>70.856627935181805</v>
+      </c>
+      <c r="X50" s="3">
+        <v>36.3922845807082</v>
+      </c>
+    </row>
+    <row r="51" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A51" s="3">
+        <v>57.4287393220986</v>
+      </c>
+      <c r="B51" s="3">
+        <v>52.849492970580997</v>
+      </c>
+      <c r="C51" s="3">
+        <v>24.844704806698299</v>
+      </c>
+      <c r="D51" s="3">
+        <v>54.156379899129199</v>
+      </c>
+      <c r="E51" s="3">
+        <v>51.640495100257901</v>
+      </c>
+      <c r="F51" s="3">
+        <v>29.638625388374201</v>
+      </c>
+      <c r="G51" s="3">
+        <v>73.424281119939494</v>
+      </c>
+      <c r="H51" s="3">
+        <v>57.3927355278093</v>
+      </c>
+      <c r="I51" s="3">
+        <v>45.149593265228901</v>
+      </c>
+      <c r="J51" s="3">
+        <v>98.531118517477793</v>
+      </c>
+      <c r="K51" s="3">
+        <v>96.628509517957497</v>
+      </c>
+      <c r="L51" s="3">
+        <v>86.855270550812804</v>
+      </c>
+      <c r="M51" s="3">
+        <v>38.035062743994303</v>
+      </c>
+      <c r="N51" s="3">
+        <v>29.088354778515001</v>
+      </c>
+      <c r="O51" s="3">
+        <v>14.995353934713799</v>
+      </c>
+      <c r="P51" s="3">
+        <v>91.040567293849307</v>
+      </c>
+      <c r="Q51" s="3">
+        <v>81.018276344650602</v>
+      </c>
+      <c r="R51" s="3">
+        <v>51.748310024064999</v>
+      </c>
+      <c r="S51" s="3">
+        <v>96.778066636362396</v>
+      </c>
+      <c r="T51" s="3">
+        <v>91.693897080623202</v>
+      </c>
+      <c r="U51" s="3">
+        <v>70.816708077669006</v>
+      </c>
+      <c r="V51" s="3">
+        <v>90.731655506271196</v>
+      </c>
+      <c r="W51" s="3">
+        <v>84.5306860711664</v>
+      </c>
+      <c r="X51" s="3">
+        <v>51.9680639020564</v>
+      </c>
+    </row>
+    <row r="52" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A52" s="3">
+        <v>49.642715902573798</v>
+      </c>
+      <c r="B52" s="3">
+        <v>45.570950831134198</v>
+      </c>
+      <c r="C52" s="3">
+        <v>23.433738370072</v>
+      </c>
+      <c r="D52" s="3">
+        <v>41.4464383789173</v>
+      </c>
+      <c r="E52" s="3">
+        <v>39.273930144472502</v>
+      </c>
+      <c r="F52" s="3">
+        <v>23.230923678607201</v>
+      </c>
+      <c r="G52" s="3">
+        <v>71.212197835541602</v>
+      </c>
+      <c r="H52" s="3">
+        <v>57.031910589663198</v>
+      </c>
+      <c r="I52" s="3">
+        <v>46.505310003034303</v>
+      </c>
+      <c r="J52" s="3">
+        <v>97.686081313864406</v>
+      </c>
+      <c r="K52" s="3">
+        <v>95.3354522148298</v>
+      </c>
+      <c r="L52" s="3">
+        <v>84.958721587396596</v>
+      </c>
+      <c r="M52" s="3">
+        <v>40.001278654531298</v>
+      </c>
+      <c r="N52" s="3">
+        <v>30.5526451268443</v>
+      </c>
+      <c r="O52" s="3">
+        <v>16.7208900534403</v>
+      </c>
+      <c r="P52" s="3">
+        <v>90.465398525573406</v>
+      </c>
+      <c r="Q52" s="3">
+        <v>81.193303607739793</v>
+      </c>
+      <c r="R52" s="3">
+        <v>54.582855648938398</v>
+      </c>
+      <c r="S52" s="3">
+        <v>95.5856256627454</v>
+      </c>
+      <c r="T52" s="3">
+        <v>90.285508454111493</v>
+      </c>
+      <c r="U52" s="3">
+        <v>70.712066364555994</v>
+      </c>
+      <c r="V52" s="3">
+        <v>89.840575149626403</v>
+      </c>
+      <c r="W52" s="3">
+        <v>84.301002799818306</v>
+      </c>
+      <c r="X52" s="3">
+        <v>54.431766859328199</v>
+      </c>
+    </row>
+    <row r="53" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A53" s="3">
+        <v>42.831439510559697</v>
+      </c>
+      <c r="B53" s="3">
+        <v>38.824917655960697</v>
+      </c>
+      <c r="C53" s="3">
+        <v>22.105150440742101</v>
+      </c>
+      <c r="D53" s="3">
+        <v>34.277095907179699</v>
+      </c>
+      <c r="E53" s="3">
+        <v>32.3493660001865</v>
+      </c>
+      <c r="F53" s="3">
+        <v>20.943202178186699</v>
+      </c>
+      <c r="G53" s="3">
+        <v>69.641702609680607</v>
+      </c>
+      <c r="H53" s="3">
+        <v>56.951553173877102</v>
+      </c>
+      <c r="I53" s="3">
+        <v>47.800374678691199</v>
+      </c>
+      <c r="J53" s="3">
+        <v>97.235084350447195</v>
+      </c>
+      <c r="K53" s="3">
+        <v>94.407256018287796</v>
+      </c>
+      <c r="L53" s="3">
+        <v>84.395658655697801</v>
+      </c>
+      <c r="M53" s="3">
+        <v>38.588415687635703</v>
+      </c>
+      <c r="N53" s="3">
+        <v>30.121252812588502</v>
+      </c>
+      <c r="O53" s="3">
+        <v>17.593264310841999</v>
+      </c>
+      <c r="P53" s="3">
+        <v>90.132276245255696</v>
+      </c>
+      <c r="Q53" s="3">
+        <v>81.719847618693905</v>
+      </c>
+      <c r="R53" s="3">
+        <v>57.820579337633497</v>
+      </c>
+      <c r="S53" s="3">
+        <v>94.386886875461002</v>
+      </c>
+      <c r="T53" s="3">
+        <v>89.329641692361506</v>
+      </c>
+      <c r="U53" s="3">
+        <v>70.9313242667818</v>
+      </c>
+      <c r="V53" s="3">
+        <v>89.188964793068095</v>
+      </c>
+      <c r="W53" s="3">
+        <v>84.299211968863403</v>
+      </c>
+      <c r="X53" s="3">
+        <v>57.582414505190897</v>
+      </c>
+    </row>
+    <row r="54" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A54" s="3">
+        <v>35.356159325651298</v>
+      </c>
+      <c r="B54" s="3">
+        <v>32.552797769715603</v>
+      </c>
+      <c r="C54" s="3">
+        <v>22.4880904265206</v>
+      </c>
+      <c r="D54" s="3">
+        <v>28.789834361829602</v>
+      </c>
+      <c r="E54" s="3">
+        <v>27.406794456495</v>
+      </c>
+      <c r="F54" s="3">
+        <v>20.150940983056302</v>
+      </c>
+      <c r="G54" s="3">
+        <v>66.493852065321803</v>
+      </c>
+      <c r="H54" s="3">
+        <v>56.2358309317964</v>
+      </c>
+      <c r="I54" s="3">
+        <v>49.172958693563899</v>
+      </c>
+      <c r="J54" s="3">
+        <v>95.873546003296696</v>
+      </c>
+      <c r="K54" s="3">
+        <v>93.109098187312895</v>
+      </c>
+      <c r="L54" s="3">
+        <v>84.3489488256225</v>
+      </c>
+      <c r="M54" s="3">
+        <v>35.912353521197403</v>
+      </c>
+      <c r="N54" s="3">
+        <v>28.3631643930193</v>
+      </c>
+      <c r="O54" s="3">
+        <v>19.715822138920199</v>
+      </c>
+      <c r="P54" s="3">
+        <v>88.493396647956601</v>
+      </c>
+      <c r="Q54" s="3">
+        <v>80.941232139561293</v>
+      </c>
+      <c r="R54" s="3">
+        <v>62.7207317462966</v>
+      </c>
+      <c r="S54" s="3">
+        <v>92.169747380611895</v>
+      </c>
+      <c r="T54" s="3">
+        <v>87.2868226847702</v>
+      </c>
+      <c r="U54" s="3">
+        <v>72.043287471000994</v>
+      </c>
+      <c r="V54" s="3">
+        <v>87.358045104060395</v>
+      </c>
+      <c r="W54" s="3">
+        <v>83.015853456505496</v>
+      </c>
+      <c r="X54" s="3">
+        <v>62.081399612046297</v>
+      </c>
+    </row>
+    <row r="55" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A55" s="3">
+        <v>33.766356008074801</v>
+      </c>
+      <c r="B55" s="3">
+        <v>32.775751843400499</v>
+      </c>
+      <c r="C55" s="3">
+        <v>29.118182645949901</v>
+      </c>
+      <c r="D55" s="3">
+        <v>28.780751329631801</v>
+      </c>
+      <c r="E55" s="3">
+        <v>28.2633156656604</v>
+      </c>
+      <c r="F55" s="3">
+        <v>26.116072578071002</v>
+      </c>
+      <c r="G55" s="3">
+        <v>62.046162376969598</v>
+      </c>
+      <c r="H55" s="3">
+        <v>56.5628205720623</v>
+      </c>
+      <c r="I55" s="3">
+        <v>53.049443186544103</v>
+      </c>
+      <c r="J55" s="3">
+        <v>92.803878524400105</v>
+      </c>
+      <c r="K55" s="3">
+        <v>91.040519333101599</v>
+      </c>
+      <c r="L55" s="3">
+        <v>86.622938757399993</v>
+      </c>
+      <c r="M55" s="3">
+        <v>35.397987640998501</v>
+      </c>
+      <c r="N55" s="3">
+        <v>32.230085121500103</v>
+      </c>
+      <c r="O55" s="3">
+        <v>28.724615225818201</v>
+      </c>
+      <c r="P55" s="3">
+        <v>85.927296544494595</v>
+      </c>
+      <c r="Q55" s="3">
+        <v>82.524784031375304</v>
+      </c>
+      <c r="R55" s="3">
+        <v>74.391757856618497</v>
+      </c>
+      <c r="S55" s="3">
+        <v>86.539828565644996</v>
+      </c>
+      <c r="T55" s="3">
+        <v>83.628651785215098</v>
+      </c>
+      <c r="U55" s="3">
+        <v>77.254093932806299</v>
+      </c>
+      <c r="V55" s="3">
+        <v>83.130502231401806</v>
+      </c>
+      <c r="W55" s="3">
+        <v>80.729123746155693</v>
+      </c>
+      <c r="X55" s="3">
+        <v>71.627539708333899</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>